<commit_message>
Add Street comparison & cross-check to Valuation Summary
Benchmark the model's valuation against published equity research
(Jefferies, UBS, Prabhudas Lilladher, Axis Capital, Motilal Oswal,
consensus). Adds a forward-multiple cross-check showing the model's
FY28E EPS (~Rs175) matches MOSL (Rs171); applying the Street's FY28E
target multiples (~40x P/E, ~25x EV/EBITDA) reproduces the ~Rs7,000
consensus, reconciling the gap vs our intrinsic blended fair value.
</commit_message>
<xml_diff>
--- a/Navin Fluorine International - Financial Model.xlsx
+++ b/Navin Fluorine International - Financial Model.xlsx
@@ -182,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -383,6 +383,18 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4056,7 +4068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N45"/>
+  <dimension ref="A1:N73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4576,8 +4588,320 @@
     <row r="43"/>
     <row r="44"/>
     <row r="45"/>
+    <row r="47">
+      <c r="A47" s="18" t="inlineStr">
+        <is>
+          <t>D.  Comparison with published equity-research (Street)</t>
+        </is>
+      </c>
+      <c r="B47" s="19" t="n"/>
+      <c r="C47" s="19" t="n"/>
+      <c r="D47" s="19" t="n"/>
+      <c r="E47" s="19" t="n"/>
+      <c r="F47" s="19" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Broker / source</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Target (Rs)</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>Valuation basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
+        <is>
+          <t>Jefferies</t>
+        </is>
+      </c>
+      <c r="B49" s="69" t="inlineStr">
+        <is>
+          <t>May-26</t>
+        </is>
+      </c>
+      <c r="C49" s="69" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D49" s="70" t="n">
+        <v>8700</v>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Premium forward multiple; CDMO/HPP ramp</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="inlineStr">
+        <is>
+          <t>Prabhudas Lilladher</t>
+        </is>
+      </c>
+      <c r="B50" s="69" t="inlineStr">
+        <is>
+          <t>Feb-26</t>
+        </is>
+      </c>
+      <c r="C50" s="69" t="inlineStr">
+        <is>
+          <t>Accumulate</t>
+        </is>
+      </c>
+      <c r="D50" s="70" t="n">
+        <v>7038</v>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Forward earnings multiple</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>Axis Capital</t>
+        </is>
+      </c>
+      <c r="B51" s="69" t="inlineStr">
+        <is>
+          <t>Feb-26</t>
+        </is>
+      </c>
+      <c r="C51" s="69" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="D51" s="70" t="n">
+        <v>7050</v>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Forward earnings multiple</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="inlineStr">
+        <is>
+          <t>UBS</t>
+        </is>
+      </c>
+      <c r="B52" s="69" t="inlineStr">
+        <is>
+          <t>Nov-25</t>
+        </is>
+      </c>
+      <c r="C52" s="69" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D52" s="70" t="n">
+        <v>7000</v>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>CDMO growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="11" t="inlineStr">
+        <is>
+          <t>Motilal Oswal</t>
+        </is>
+      </c>
+      <c r="B53" s="69" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="C53" s="69" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="D53" s="70" t="n">
+        <v>6840</v>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>~40x FY28E EPS (Rs171); ~25x FY28E EV/EBITDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="11" t="inlineStr">
+        <is>
+          <t>Consensus (27 analysts)</t>
+        </is>
+      </c>
+      <c r="B54" s="69" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="C54" s="69" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D54" s="70" t="n">
+        <v>7316</v>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>12-month average target</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>Street average target (excl. consensus row)</t>
+        </is>
+      </c>
+      <c r="D55" s="71">
+        <f>AVERAGE(D49:D53)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>This model - blended fair value</t>
+        </is>
+      </c>
+      <c r="D56" s="72">
+        <f>D35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="18" t="inlineStr">
+        <is>
+          <t>Cross-check: apply Street FY28E target multiples to THIS model's forecasts</t>
+        </is>
+      </c>
+      <c r="B58" s="19" t="n"/>
+      <c r="C58" s="19" t="n"/>
+      <c r="D58" s="19" t="n"/>
+      <c r="E58" s="19" t="n"/>
+      <c r="F58" s="19" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="11" t="inlineStr">
+        <is>
+          <t>This model FY28E EPS (Rs)  [MOSL: Rs171]</t>
+        </is>
+      </c>
+      <c r="B59" s="16">
+        <f>'Profit &amp; Loss'!I22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>This model FY28E EBITDA (Rs Cr)</t>
+        </is>
+      </c>
+      <c r="B60" s="30">
+        <f>'Profit &amp; Loss'!I10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="11" t="inlineStr">
+        <is>
+          <t>Target P/E multiple (Street, x)</t>
+        </is>
+      </c>
+      <c r="B61" s="45" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>Target EV/EBITDA multiple (Street, x)</t>
+        </is>
+      </c>
+      <c r="B62" s="45" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>Implied value/share - 40x FY28E EPS</t>
+        </is>
+      </c>
+      <c r="B63" s="55">
+        <f>B61*B59</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>Implied value/share - 25x FY28E EV/EBITDA</t>
+        </is>
+      </c>
+      <c r="B64" s="55">
+        <f>(B62*B60-B22)/B23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>Street-aligned fair value (avg of the two)</t>
+        </is>
+      </c>
+      <c r="B65" s="41">
+        <f>AVERAGE(B63:B64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67" ht="110" customHeight="1">
+      <c r="A67" s="58" t="inlineStr">
+        <is>
+          <t>Reconciliation: This model's FY28E EPS (~Rs175) is in line with Motilal Oswal's Rs171, confirming the forecasts agree with the Street. Applying the Street's FY28E target multiples (~40x P/E, ~25x EV/EBITDA) to these forecasts yields ~Rs7,000/share - consistent with the consensus target of ~Rs7,316. The difference versus our blended fair value (~Rs4,450) is therefore NOT a forecast disagreement but a deliberate valuation-discipline choice: (i) horizon - the Street rolls valuation to FY28E whereas our DCF/relative anchors to FY27E and intrinsic cash flows; and (ii) multiple - the Street assigns premium target multiples for the franchise's scarcity/quality versus our peer-median and WACC-based anchors. Bottom line: on the Street's forward, premium-multiple framework the stock is fairly valued (~Rs7,000-7,300); on a disciplined intrinsic/peer-relative basis it looks expensive (~Rs4,450). We flag the stock as fully valued, with the Street pricing in a long runway of execution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A67:N73"/>
     <mergeCell ref="A40:N45"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Enhance model: segment revenue build, cash-allocation sweep, scenarios, dual-terminal DCF, charts
- Bottom-up revenue by segment (HPP/Refrigerants, Specialty Chemicals,
  CDMO/CRAMS) feeding the P&L, anchored to disclosed Q3FY26 mix.
- Capital-allocation cash sweep: surplus over a 15%-of-revenue buffer
  returned via dividend/buyback, removing the unrealistic cash build-up
  and lifting ROE to ~18-23% and ROIC to ~18-25%.
- DCF terminal value cross-check via exit EV/EBITDA multiple; intrinsic
  now the average of Gordon-growth and exit-multiple methods.
- Bull/Base/Bear scenario analysis on FY28E EPS multiples.
- Charts: revenue & EBITDA, PAT, FCFF, and a valuation football field.
- All statements still fully integrated; balance sheet balances (0).
</commit_message>
<xml_diff>
--- a/Navin Fluorine International - Financial Model.xlsx
+++ b/Navin Fluorine International - Financial Model.xlsx
@@ -35,7 +35,7 @@
     <numFmt numFmtId="168" formatCode="0.0%"/>
     <numFmt numFmtId="169" formatCode="0.000"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -131,6 +131,12 @@
       <color rgb="00404040"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00595959"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -182,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -203,7 +209,7 @@
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -249,7 +255,7 @@
     <xf numFmtId="10" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -396,6 +402,27 @@
     <xf numFmtId="3" fontId="12" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -470,6 +497,556 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Revenue &amp; EBITDA (Rs Cr), FY21-FY33</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Summary'!A20</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Summary'!$B$19:$N$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Summary'!$B$20:$N$20</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Summary'!A21</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Summary'!$B$19:$N$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Summary'!$B$21:$N$21</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>PAT (Rs Cr), FY21-FY33</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Summary'!A24</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Summary'!$B$19:$N$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Summary'!$B$24:$N$24</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Navin Fluorine - valuation football field (Rs/share)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Valuation Summary'!$A$87:$A$95</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Valuation Summary'!$B$87:$B$95</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>FCFF (Rs Cr), FY27-FY33</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'DCF'!$B$19:$H$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'DCF'!$B$26</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'DCF'!$B$19:$H$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'DCF'!$C$26</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'DCF'!$B$19:$H$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'DCF'!$D$26</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'DCF'!$B$19:$H$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'DCF'!$E$26</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'DCF'!$B$19:$H$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'DCF'!$F$26</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'DCF'!$B$19:$H$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'DCF'!$G$26</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'DCF'!$B$19:$H$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'DCF'!$H$26</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>55</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>74</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>43</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1682,6 +2259,7 @@
     <mergeCell ref="A36:N36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1691,7 +2269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:N42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2024,31 +2602,31 @@
         <f>'Balance Sheet'!G5</f>
         <v/>
       </c>
-      <c r="H8" s="8">
+      <c r="H8" s="77">
         <f>H5-H6+H7</f>
         <v/>
       </c>
-      <c r="I8" s="8">
+      <c r="I8" s="77">
         <f>I5-I6+I7</f>
         <v/>
       </c>
-      <c r="J8" s="8">
+      <c r="J8" s="77">
         <f>J5-J6+J7</f>
         <v/>
       </c>
-      <c r="K8" s="8">
+      <c r="K8" s="77">
         <f>K5-K6+K7</f>
         <v/>
       </c>
-      <c r="L8" s="8">
+      <c r="L8" s="77">
         <f>L5-L6+L7</f>
         <v/>
       </c>
-      <c r="M8" s="8">
+      <c r="M8" s="77">
         <f>M5-M6+M7</f>
         <v/>
       </c>
-      <c r="N8" s="8">
+      <c r="N8" s="77">
         <f>N5-N6+N7</f>
         <v/>
       </c>
@@ -2465,32 +3043,32 @@
         <f>G17+G18+G20-G21</f>
         <v/>
       </c>
-      <c r="H19" s="13">
-        <f>H18*Assumptions!H13</f>
-        <v/>
-      </c>
-      <c r="I19" s="13">
-        <f>I18*Assumptions!I13</f>
-        <v/>
-      </c>
-      <c r="J19" s="13">
-        <f>J18*Assumptions!J13</f>
-        <v/>
-      </c>
-      <c r="K19" s="13">
-        <f>K18*Assumptions!K13</f>
-        <v/>
-      </c>
-      <c r="L19" s="13">
-        <f>L18*Assumptions!L13</f>
-        <v/>
-      </c>
-      <c r="M19" s="13">
-        <f>M18*Assumptions!M13</f>
-        <v/>
-      </c>
-      <c r="N19" s="13">
-        <f>N18*Assumptions!N13</f>
+      <c r="H19" s="16">
+        <f>H41</f>
+        <v/>
+      </c>
+      <c r="I19" s="16">
+        <f>I41</f>
+        <v/>
+      </c>
+      <c r="J19" s="16">
+        <f>J41</f>
+        <v/>
+      </c>
+      <c r="K19" s="16">
+        <f>K41</f>
+        <v/>
+      </c>
+      <c r="L19" s="16">
+        <f>L41</f>
+        <v/>
+      </c>
+      <c r="M19" s="16">
+        <f>M41</f>
+        <v/>
+      </c>
+      <c r="N19" s="16">
+        <f>N41</f>
         <v/>
       </c>
     </row>
@@ -2568,31 +3146,31 @@
         <f>'Balance Sheet'!G17</f>
         <v/>
       </c>
-      <c r="H21" s="8">
+      <c r="H21" s="77">
         <f>H17+H18-H19+H20</f>
         <v/>
       </c>
-      <c r="I21" s="8">
+      <c r="I21" s="77">
         <f>I17+I18-I19+I20</f>
         <v/>
       </c>
-      <c r="J21" s="8">
+      <c r="J21" s="77">
         <f>J17+J18-J19+J20</f>
         <v/>
       </c>
-      <c r="K21" s="8">
+      <c r="K21" s="77">
         <f>K17+K18-K19+K20</f>
         <v/>
       </c>
-      <c r="L21" s="8">
+      <c r="L21" s="77">
         <f>L17+L18-L19+L20</f>
         <v/>
       </c>
-      <c r="M21" s="8">
+      <c r="M21" s="77">
         <f>M17+M18-M19+M20</f>
         <v/>
       </c>
-      <c r="N21" s="8">
+      <c r="N21" s="77">
         <f>N17+N18-N19+N20</f>
         <v/>
       </c>
@@ -2859,56 +3437,489 @@
           <t>Net debt / (net cash)</t>
         </is>
       </c>
-      <c r="B28" s="8">
+      <c r="B28" s="77">
         <f>B26-B27</f>
         <v/>
       </c>
-      <c r="C28" s="8">
+      <c r="C28" s="77">
         <f>C26-C27</f>
         <v/>
       </c>
-      <c r="D28" s="8">
+      <c r="D28" s="77">
         <f>D26-D27</f>
         <v/>
       </c>
-      <c r="E28" s="8">
+      <c r="E28" s="77">
         <f>E26-E27</f>
         <v/>
       </c>
-      <c r="F28" s="8">
+      <c r="F28" s="77">
         <f>F26-F27</f>
         <v/>
       </c>
-      <c r="G28" s="8">
+      <c r="G28" s="77">
         <f>G26-G27</f>
         <v/>
       </c>
-      <c r="H28" s="8">
+      <c r="H28" s="77">
         <f>H26-H27</f>
         <v/>
       </c>
-      <c r="I28" s="8">
+      <c r="I28" s="77">
         <f>I26-I27</f>
         <v/>
       </c>
-      <c r="J28" s="8">
+      <c r="J28" s="77">
         <f>J26-J27</f>
         <v/>
       </c>
-      <c r="K28" s="8">
+      <c r="K28" s="77">
         <f>K26-K27</f>
         <v/>
       </c>
-      <c r="L28" s="8">
+      <c r="L28" s="77">
         <f>L26-L27</f>
         <v/>
       </c>
-      <c r="M28" s="8">
+      <c r="M28" s="77">
         <f>M26-M27</f>
         <v/>
       </c>
-      <c r="N28" s="8">
+      <c r="N28" s="77">
         <f>N26-N27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="18" t="inlineStr">
+        <is>
+          <t>Capital allocation &amp; cash sweep</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="n"/>
+      <c r="C30" s="19" t="n"/>
+      <c r="D30" s="19" t="n"/>
+      <c r="E30" s="19" t="n"/>
+      <c r="F30" s="19" t="n"/>
+      <c r="G30" s="19" t="n"/>
+      <c r="H30" s="19" t="n"/>
+      <c r="I30" s="19" t="n"/>
+      <c r="J30" s="19" t="n"/>
+      <c r="K30" s="19" t="n"/>
+      <c r="L30" s="19" t="n"/>
+      <c r="M30" s="19" t="n"/>
+      <c r="N30" s="19" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>Target cash &amp; investments (% of revenue)</t>
+        </is>
+      </c>
+      <c r="H31" s="51" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="I31" s="51" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J31" s="51" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K31" s="51" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="L31" s="51" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="M31" s="51" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="N31" s="51" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>Target cash &amp; investments (Rs Cr)</t>
+        </is>
+      </c>
+      <c r="H32" s="13">
+        <f>H31*'Profit &amp; Loss'!H4</f>
+        <v/>
+      </c>
+      <c r="I32" s="13">
+        <f>I31*'Profit &amp; Loss'!I4</f>
+        <v/>
+      </c>
+      <c r="J32" s="13">
+        <f>J31*'Profit &amp; Loss'!J4</f>
+        <v/>
+      </c>
+      <c r="K32" s="13">
+        <f>K31*'Profit &amp; Loss'!K4</f>
+        <v/>
+      </c>
+      <c r="L32" s="13">
+        <f>L31*'Profit &amp; Loss'!L4</f>
+        <v/>
+      </c>
+      <c r="M32" s="13">
+        <f>M31*'Profit &amp; Loss'!M4</f>
+        <v/>
+      </c>
+      <c r="N32" s="13">
+        <f>N31*'Profit &amp; Loss'!N4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>Opening cash &amp; investments</t>
+        </is>
+      </c>
+      <c r="H33" s="16">
+        <f>'Balance Sheet'!G11</f>
+        <v/>
+      </c>
+      <c r="I33" s="16">
+        <f>'Balance Sheet'!H11</f>
+        <v/>
+      </c>
+      <c r="J33" s="16">
+        <f>'Balance Sheet'!I11</f>
+        <v/>
+      </c>
+      <c r="K33" s="16">
+        <f>'Balance Sheet'!J11</f>
+        <v/>
+      </c>
+      <c r="L33" s="16">
+        <f>'Balance Sheet'!K11</f>
+        <v/>
+      </c>
+      <c r="M33" s="16">
+        <f>'Balance Sheet'!L11</f>
+        <v/>
+      </c>
+      <c r="N33" s="16">
+        <f>'Balance Sheet'!M11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>Add: PAT</t>
+        </is>
+      </c>
+      <c r="H34" s="16">
+        <f>'Profit &amp; Loss'!H21</f>
+        <v/>
+      </c>
+      <c r="I34" s="16">
+        <f>'Profit &amp; Loss'!I21</f>
+        <v/>
+      </c>
+      <c r="J34" s="16">
+        <f>'Profit &amp; Loss'!J21</f>
+        <v/>
+      </c>
+      <c r="K34" s="16">
+        <f>'Profit &amp; Loss'!K21</f>
+        <v/>
+      </c>
+      <c r="L34" s="16">
+        <f>'Profit &amp; Loss'!L21</f>
+        <v/>
+      </c>
+      <c r="M34" s="16">
+        <f>'Profit &amp; Loss'!M21</f>
+        <v/>
+      </c>
+      <c r="N34" s="16">
+        <f>'Profit &amp; Loss'!N21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>Add: Depreciation</t>
+        </is>
+      </c>
+      <c r="H35" s="16">
+        <f>'Profit &amp; Loss'!H12</f>
+        <v/>
+      </c>
+      <c r="I35" s="16">
+        <f>'Profit &amp; Loss'!I12</f>
+        <v/>
+      </c>
+      <c r="J35" s="16">
+        <f>'Profit &amp; Loss'!J12</f>
+        <v/>
+      </c>
+      <c r="K35" s="16">
+        <f>'Profit &amp; Loss'!K12</f>
+        <v/>
+      </c>
+      <c r="L35" s="16">
+        <f>'Profit &amp; Loss'!L12</f>
+        <v/>
+      </c>
+      <c r="M35" s="16">
+        <f>'Profit &amp; Loss'!M12</f>
+        <v/>
+      </c>
+      <c r="N35" s="16">
+        <f>'Profit &amp; Loss'!N12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>Less: Increase in net working capital</t>
+        </is>
+      </c>
+      <c r="H36" s="16">
+        <f>'Working Capital Schedule'!H12</f>
+        <v/>
+      </c>
+      <c r="I36" s="16">
+        <f>'Working Capital Schedule'!I12</f>
+        <v/>
+      </c>
+      <c r="J36" s="16">
+        <f>'Working Capital Schedule'!J12</f>
+        <v/>
+      </c>
+      <c r="K36" s="16">
+        <f>'Working Capital Schedule'!K12</f>
+        <v/>
+      </c>
+      <c r="L36" s="16">
+        <f>'Working Capital Schedule'!L12</f>
+        <v/>
+      </c>
+      <c r="M36" s="16">
+        <f>'Working Capital Schedule'!M12</f>
+        <v/>
+      </c>
+      <c r="N36" s="16">
+        <f>'Working Capital Schedule'!N12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>Less: Capital expenditure</t>
+        </is>
+      </c>
+      <c r="H37" s="16">
+        <f>Assumptions!H11</f>
+        <v/>
+      </c>
+      <c r="I37" s="16">
+        <f>Assumptions!I11</f>
+        <v/>
+      </c>
+      <c r="J37" s="16">
+        <f>Assumptions!J11</f>
+        <v/>
+      </c>
+      <c r="K37" s="16">
+        <f>Assumptions!K11</f>
+        <v/>
+      </c>
+      <c r="L37" s="16">
+        <f>Assumptions!L11</f>
+        <v/>
+      </c>
+      <c r="M37" s="16">
+        <f>Assumptions!M11</f>
+        <v/>
+      </c>
+      <c r="N37" s="16">
+        <f>Assumptions!N11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>Add: Change in borrowings</t>
+        </is>
+      </c>
+      <c r="H38" s="13">
+        <f>H12-H11</f>
+        <v/>
+      </c>
+      <c r="I38" s="13">
+        <f>I12-I11</f>
+        <v/>
+      </c>
+      <c r="J38" s="13">
+        <f>J12-J11</f>
+        <v/>
+      </c>
+      <c r="K38" s="13">
+        <f>K12-K11</f>
+        <v/>
+      </c>
+      <c r="L38" s="13">
+        <f>L12-L11</f>
+        <v/>
+      </c>
+      <c r="M38" s="13">
+        <f>M12-M11</f>
+        <v/>
+      </c>
+      <c r="N38" s="13">
+        <f>N12-N11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Cash available before distribution</t>
+        </is>
+      </c>
+      <c r="H39" s="77">
+        <f>H33+H34+H35-H36-H37+H38+H20</f>
+        <v/>
+      </c>
+      <c r="I39" s="77">
+        <f>I33+I34+I35-I36-I37+I38+I20</f>
+        <v/>
+      </c>
+      <c r="J39" s="77">
+        <f>J33+J34+J35-J36-J37+J38+J20</f>
+        <v/>
+      </c>
+      <c r="K39" s="77">
+        <f>K33+K34+K35-K36-K37+K38+K20</f>
+        <v/>
+      </c>
+      <c r="L39" s="77">
+        <f>L33+L34+L35-L36-L37+L38+L20</f>
+        <v/>
+      </c>
+      <c r="M39" s="77">
+        <f>M33+M34+M35-M36-M37+M38+M20</f>
+        <v/>
+      </c>
+      <c r="N39" s="77">
+        <f>N33+N34+N35-N36-N37+N38+N20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>Base dividend (payout x PAT)</t>
+        </is>
+      </c>
+      <c r="H40" s="13">
+        <f>'Profit &amp; Loss'!H21*Assumptions!H13</f>
+        <v/>
+      </c>
+      <c r="I40" s="13">
+        <f>'Profit &amp; Loss'!I21*Assumptions!I13</f>
+        <v/>
+      </c>
+      <c r="J40" s="13">
+        <f>'Profit &amp; Loss'!J21*Assumptions!J13</f>
+        <v/>
+      </c>
+      <c r="K40" s="13">
+        <f>'Profit &amp; Loss'!K21*Assumptions!K13</f>
+        <v/>
+      </c>
+      <c r="L40" s="13">
+        <f>'Profit &amp; Loss'!L21*Assumptions!L13</f>
+        <v/>
+      </c>
+      <c r="M40" s="13">
+        <f>'Profit &amp; Loss'!M21*Assumptions!M13</f>
+        <v/>
+      </c>
+      <c r="N40" s="13">
+        <f>'Profit &amp; Loss'!N21*Assumptions!N13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Total distribution (dividend + buyback/special)</t>
+        </is>
+      </c>
+      <c r="H41" s="77">
+        <f>MAX(H40,H39-H32)</f>
+        <v/>
+      </c>
+      <c r="I41" s="77">
+        <f>MAX(I40,I39-I32)</f>
+        <v/>
+      </c>
+      <c r="J41" s="77">
+        <f>MAX(J40,J39-J32)</f>
+        <v/>
+      </c>
+      <c r="K41" s="77">
+        <f>MAX(K40,K39-K32)</f>
+        <v/>
+      </c>
+      <c r="L41" s="77">
+        <f>MAX(L40,L39-L32)</f>
+        <v/>
+      </c>
+      <c r="M41" s="77">
+        <f>MAX(M40,M39-M32)</f>
+        <v/>
+      </c>
+      <c r="N41" s="77">
+        <f>MAX(N40,N39-N32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>Closing cash &amp; investments (= BS)</t>
+        </is>
+      </c>
+      <c r="H42" s="15">
+        <f>H39-H41</f>
+        <v/>
+      </c>
+      <c r="I42" s="15">
+        <f>I39-I41</f>
+        <v/>
+      </c>
+      <c r="J42" s="15">
+        <f>J39-J41</f>
+        <v/>
+      </c>
+      <c r="K42" s="15">
+        <f>K39-K41</f>
+        <v/>
+      </c>
+      <c r="L42" s="15">
+        <f>L39-L41</f>
+        <v/>
+      </c>
+      <c r="M42" s="15">
+        <f>M39-M41</f>
+        <v/>
+      </c>
+      <c r="N42" s="15">
+        <f>N39-N41</f>
         <v/>
       </c>
     </row>
@@ -4068,7 +5079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N73"/>
+  <dimension ref="A1:N95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4153,7 +5164,7 @@
         </is>
       </c>
       <c r="B7" s="54">
-        <f>DCF!B38</f>
+        <f>DCF!B77</f>
         <v/>
       </c>
     </row>
@@ -4899,12 +5910,232 @@
     <row r="71"/>
     <row r="72"/>
     <row r="73"/>
+    <row r="75">
+      <c r="A75" s="18" t="inlineStr">
+        <is>
+          <t>E.  Scenario analysis (fair value, Rs/share)</t>
+        </is>
+      </c>
+      <c r="B75" s="19" t="n"/>
+      <c r="C75" s="19" t="n"/>
+      <c r="D75" s="19" t="n"/>
+      <c r="E75" s="19" t="n"/>
+      <c r="F75" s="19" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>FY28E EPS x mult</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Fair value (Rs)</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>vs CMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="11" t="inlineStr">
+        <is>
+          <t>Bull  (45x FY28E EPS; faster CDMO/HPP)</t>
+        </is>
+      </c>
+      <c r="B77" s="73" t="n">
+        <v>45</v>
+      </c>
+      <c r="C77" s="55">
+        <f>B77*B59</f>
+        <v/>
+      </c>
+      <c r="D77" s="27">
+        <f>C77/DCF!B39-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="inlineStr">
+        <is>
+          <t>Base  (40x FY28E EPS; in line with MOSL)</t>
+        </is>
+      </c>
+      <c r="B78" s="73" t="n">
+        <v>40</v>
+      </c>
+      <c r="C78" s="55">
+        <f>B78*B59</f>
+        <v/>
+      </c>
+      <c r="D78" s="27">
+        <f>C78/DCF!B39-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="11" t="inlineStr">
+        <is>
+          <t>Bear  (32x FY28E EPS; peer-median de-rating)</t>
+        </is>
+      </c>
+      <c r="B79" s="73" t="n">
+        <v>32</v>
+      </c>
+      <c r="C79" s="55">
+        <f>B79*B59</f>
+        <v/>
+      </c>
+      <c r="D79" s="27">
+        <f>C79/DCF!B39-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="inlineStr">
+        <is>
+          <t>DCF intrinsic (Gordon + exit-multiple avg)</t>
+        </is>
+      </c>
+      <c r="C80" s="74">
+        <f>DCF!B77</f>
+        <v/>
+      </c>
+      <c r="D80" s="27">
+        <f>C80/DCF!B39-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81" ht="44" customHeight="1">
+      <c r="A81" s="53" t="inlineStr">
+        <is>
+          <t>Note: Bull/Base/Bear apply forward P/E multiples to this model's FY28E EPS (~Rs175). Base (40x) mirrors the Street's framework; the DCF row is the disciplined intrinsic anchor. The spread frames the risk/reward around the current price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="86">
+      <c r="A86" s="75" t="inlineStr">
+        <is>
+          <t>Valuation methods (Rs/share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="11" t="inlineStr">
+        <is>
+          <t>DCF (intrinsic)</t>
+        </is>
+      </c>
+      <c r="B87" s="56">
+        <f>DCF!B77</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="11" t="inlineStr">
+        <is>
+          <t>Relative P/E</t>
+        </is>
+      </c>
+      <c r="B88" s="56">
+        <f>B25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="11" t="inlineStr">
+        <is>
+          <t>Relative EV/EBITDA</t>
+        </is>
+      </c>
+      <c r="B89" s="56">
+        <f>B26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="11" t="inlineStr">
+        <is>
+          <t>Relative EV/Sales</t>
+        </is>
+      </c>
+      <c r="B90" s="56">
+        <f>B27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="11" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="B91" s="56">
+        <f>C77</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="11" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="B92" s="56">
+        <f>C78</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="11" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="B93" s="56">
+        <f>C79</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="11" t="inlineStr">
+        <is>
+          <t>Blended target</t>
+        </is>
+      </c>
+      <c r="B94" s="56">
+        <f>D35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="11" t="inlineStr">
+        <is>
+          <t>Current price</t>
+        </is>
+      </c>
+      <c r="B95" s="56">
+        <f>DCF!B39</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A81:N83"/>
     <mergeCell ref="A67:N73"/>
     <mergeCell ref="A40:N45"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4914,7 +6145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N50"/>
+  <dimension ref="A1:N77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4975,7 +6206,7 @@
           <t>Risk-free rate (Rf, India 10Y G-sec)</t>
         </is>
       </c>
-      <c r="B5" s="24" t="n">
+      <c r="B5" s="76" t="n">
         <v>0.068</v>
       </c>
     </row>
@@ -4985,7 +6216,7 @@
           <t>Equity risk premium (ERP)</t>
         </is>
       </c>
-      <c r="B6" s="24" t="n">
+      <c r="B6" s="76" t="n">
         <v>0.06</v>
       </c>
     </row>
@@ -5017,7 +6248,7 @@
           <t>Pre-tax cost of debt (Kd)</t>
         </is>
       </c>
-      <c r="B9" s="24" t="n">
+      <c r="B9" s="76" t="n">
         <v>0.075</v>
       </c>
     </row>
@@ -5027,7 +6258,7 @@
           <t>Marginal tax rate</t>
         </is>
       </c>
-      <c r="B10" s="24" t="n">
+      <c r="B10" s="76" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -5102,7 +6333,7 @@
           <t>Terminal growth rate (g)</t>
         </is>
       </c>
-      <c r="B17" s="24" t="n">
+      <c r="B17" s="76" t="n">
         <v>0.055</v>
       </c>
     </row>
@@ -5224,31 +6455,31 @@
           <t>NOPAT</t>
         </is>
       </c>
-      <c r="B22" s="8">
+      <c r="B22" s="77">
         <f>B20-B21</f>
         <v/>
       </c>
-      <c r="C22" s="8">
+      <c r="C22" s="77">
         <f>C20-C21</f>
         <v/>
       </c>
-      <c r="D22" s="8">
+      <c r="D22" s="77">
         <f>D20-D21</f>
         <v/>
       </c>
-      <c r="E22" s="8">
+      <c r="E22" s="77">
         <f>E20-E21</f>
         <v/>
       </c>
-      <c r="F22" s="8">
+      <c r="F22" s="77">
         <f>F20-F21</f>
         <v/>
       </c>
-      <c r="G22" s="8">
+      <c r="G22" s="77">
         <f>G20-G21</f>
         <v/>
       </c>
-      <c r="H22" s="8">
+      <c r="H22" s="77">
         <f>H20-H21</f>
         <v/>
       </c>
@@ -5462,31 +6693,31 @@
           <t>PV of FCFF</t>
         </is>
       </c>
-      <c r="B29" s="8">
+      <c r="B29" s="77">
         <f>B26*B28</f>
         <v/>
       </c>
-      <c r="C29" s="8">
+      <c r="C29" s="77">
         <f>C26*C28</f>
         <v/>
       </c>
-      <c r="D29" s="8">
+      <c r="D29" s="77">
         <f>D26*D28</f>
         <v/>
       </c>
-      <c r="E29" s="8">
+      <c r="E29" s="77">
         <f>E26*E28</f>
         <v/>
       </c>
-      <c r="F29" s="8">
+      <c r="F29" s="77">
         <f>F26*F28</f>
         <v/>
       </c>
-      <c r="G29" s="8">
+      <c r="G29" s="77">
         <f>G26*G28</f>
         <v/>
       </c>
-      <c r="H29" s="8">
+      <c r="H29" s="77">
         <f>H26*H28</f>
         <v/>
       </c>
@@ -5497,7 +6728,7 @@
           <t>PV of explicit FCFF (FY27-FY33)</t>
         </is>
       </c>
-      <c r="B31" s="8">
+      <c r="B31" s="77">
         <f>SUM(B29:H29)</f>
         <v/>
       </c>
@@ -5552,7 +6783,7 @@
           <t>Equity value</t>
         </is>
       </c>
-      <c r="B36" s="8">
+      <c r="B36" s="77">
         <f>B34-B35</f>
         <v/>
       </c>
@@ -5771,8 +7002,105 @@
         <v/>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" s="18" t="inlineStr">
+        <is>
+          <t>Terminal value cross-check - exit EV/EBITDA multiple</t>
+        </is>
+      </c>
+      <c r="B69" s="19" t="n"/>
+      <c r="C69" s="19" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="inlineStr">
+        <is>
+          <t>Exit EV/EBITDA multiple (x)</t>
+        </is>
+      </c>
+      <c r="B70" s="45" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="11" t="inlineStr">
+        <is>
+          <t>Terminal-year (FY33) EBITDA</t>
+        </is>
+      </c>
+      <c r="B71" s="30">
+        <f>'Profit &amp; Loss'!N10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="inlineStr">
+        <is>
+          <t>Terminal value (exit multiple)</t>
+        </is>
+      </c>
+      <c r="B72" s="68">
+        <f>B70*B71</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="11" t="inlineStr">
+        <is>
+          <t>PV of terminal value (exit)</t>
+        </is>
+      </c>
+      <c r="B73" s="68">
+        <f>B72*H28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>Enterprise value (exit method)</t>
+        </is>
+      </c>
+      <c r="B74" s="78">
+        <f>B31+B73</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="11" t="inlineStr">
+        <is>
+          <t>Equity value (exit method)</t>
+        </is>
+      </c>
+      <c r="B75" s="68">
+        <f>B74-B35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>Intrinsic value/share - exit multiple (Rs)</t>
+        </is>
+      </c>
+      <c r="B76" s="41">
+        <f>B75/B37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>DCF value (avg of Gordon-growth &amp; exit-multiple)</t>
+        </is>
+      </c>
+      <c r="B77" s="41">
+        <f>AVERAGE(B38,B76)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -7258,32 +8586,32 @@
       <c r="G4" s="7" t="n">
         <v>3314</v>
       </c>
-      <c r="H4" s="8">
-        <f>G4*(1+Assumptions!H5)</f>
-        <v/>
-      </c>
-      <c r="I4" s="8">
-        <f>H4*(1+Assumptions!I5)</f>
-        <v/>
-      </c>
-      <c r="J4" s="8">
-        <f>I4*(1+Assumptions!J5)</f>
-        <v/>
-      </c>
-      <c r="K4" s="8">
-        <f>J4*(1+Assumptions!K5)</f>
-        <v/>
-      </c>
-      <c r="L4" s="8">
-        <f>K4*(1+Assumptions!L5)</f>
-        <v/>
-      </c>
-      <c r="M4" s="8">
-        <f>L4*(1+Assumptions!M5)</f>
-        <v/>
-      </c>
-      <c r="N4" s="8">
-        <f>M4*(1+Assumptions!N5)</f>
+      <c r="H4" s="22">
+        <f>Assumptions!H44</f>
+        <v/>
+      </c>
+      <c r="I4" s="22">
+        <f>Assumptions!I44</f>
+        <v/>
+      </c>
+      <c r="J4" s="22">
+        <f>Assumptions!J44</f>
+        <v/>
+      </c>
+      <c r="K4" s="22">
+        <f>Assumptions!K44</f>
+        <v/>
+      </c>
+      <c r="L4" s="22">
+        <f>Assumptions!L44</f>
+        <v/>
+      </c>
+      <c r="M4" s="22">
+        <f>Assumptions!M44</f>
+        <v/>
+      </c>
+      <c r="N4" s="22">
+        <f>Assumptions!N44</f>
         <v/>
       </c>
     </row>
@@ -7314,31 +8642,31 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>IF(G4=0,"",H4/G4-1)</f>
+        <f>IF(Assumptions!G44=0,"",Assumptions!H44/Assumptions!G44-1)</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>IF(H4=0,"",I4/H4-1)</f>
+        <f>IF(Assumptions!H44=0,"",Assumptions!I44/Assumptions!H44-1)</f>
         <v/>
       </c>
       <c r="J5" s="10">
-        <f>IF(I4=0,"",J4/I4-1)</f>
+        <f>IF(Assumptions!I44=0,"",Assumptions!J44/Assumptions!I44-1)</f>
         <v/>
       </c>
       <c r="K5" s="10">
-        <f>IF(J4=0,"",K4/J4-1)</f>
+        <f>IF(Assumptions!J44=0,"",Assumptions!K44/Assumptions!J44-1)</f>
         <v/>
       </c>
       <c r="L5" s="10">
-        <f>IF(K4=0,"",L4/K4-1)</f>
+        <f>IF(Assumptions!K44=0,"",Assumptions!L44/Assumptions!K44-1)</f>
         <v/>
       </c>
       <c r="M5" s="10">
-        <f>IF(L4=0,"",M4/L4-1)</f>
+        <f>IF(Assumptions!L44=0,"",Assumptions!M44/Assumptions!L44-1)</f>
         <v/>
       </c>
       <c r="N5" s="10">
-        <f>IF(M4=0,"",N4/M4-1)</f>
+        <f>IF(Assumptions!M44=0,"",Assumptions!N44/Assumptions!M44-1)</f>
         <v/>
       </c>
     </row>
@@ -7737,55 +9065,55 @@
           <t>EBIT</t>
         </is>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="77">
         <f>B10-B12</f>
         <v/>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="77">
         <f>C10-C12</f>
         <v/>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="77">
         <f>D10-D12</f>
         <v/>
       </c>
-      <c r="E13" s="8">
+      <c r="E13" s="77">
         <f>E10-E12</f>
         <v/>
       </c>
-      <c r="F13" s="8">
+      <c r="F13" s="77">
         <f>F10-F12</f>
         <v/>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="77">
         <f>G10-G12</f>
         <v/>
       </c>
-      <c r="H13" s="8">
+      <c r="H13" s="77">
         <f>H10-H12</f>
         <v/>
       </c>
-      <c r="I13" s="8">
+      <c r="I13" s="77">
         <f>I10-I12</f>
         <v/>
       </c>
-      <c r="J13" s="8">
+      <c r="J13" s="77">
         <f>J10-J12</f>
         <v/>
       </c>
-      <c r="K13" s="8">
+      <c r="K13" s="77">
         <f>K10-K12</f>
         <v/>
       </c>
-      <c r="L13" s="8">
+      <c r="L13" s="77">
         <f>L10-L12</f>
         <v/>
       </c>
-      <c r="M13" s="8">
+      <c r="M13" s="77">
         <f>M10-M12</f>
         <v/>
       </c>
-      <c r="N13" s="8">
+      <c r="N13" s="77">
         <f>N10-N12</f>
         <v/>
       </c>
@@ -10052,55 +11380,55 @@
           <t>Net increase / (decrease) in cash &amp; investments</t>
         </is>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="77">
         <f>B8+B11+B17</f>
         <v/>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="77">
         <f>C8+C11+C17</f>
         <v/>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="77">
         <f>D8+D11+D17</f>
         <v/>
       </c>
-      <c r="E19" s="8">
+      <c r="E19" s="77">
         <f>E8+E11+E17</f>
         <v/>
       </c>
-      <c r="F19" s="8">
+      <c r="F19" s="77">
         <f>F8+F11+F17</f>
         <v/>
       </c>
-      <c r="G19" s="8">
+      <c r="G19" s="77">
         <f>G8+G11+G17</f>
         <v/>
       </c>
-      <c r="H19" s="8">
+      <c r="H19" s="77">
         <f>H8+H11+H17</f>
         <v/>
       </c>
-      <c r="I19" s="8">
+      <c r="I19" s="77">
         <f>I8+I11+I17</f>
         <v/>
       </c>
-      <c r="J19" s="8">
+      <c r="J19" s="77">
         <f>J8+J11+J17</f>
         <v/>
       </c>
-      <c r="K19" s="8">
+      <c r="K19" s="77">
         <f>K8+K11+K17</f>
         <v/>
       </c>
-      <c r="L19" s="8">
+      <c r="L19" s="77">
         <f>L8+L11+L17</f>
         <v/>
       </c>
-      <c r="M19" s="8">
+      <c r="M19" s="77">
         <f>M8+M11+M17</f>
         <v/>
       </c>
-      <c r="N19" s="8">
+      <c r="N19" s="77">
         <f>N8+N11+N17</f>
         <v/>
       </c>
@@ -10210,7 +11538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N33"/>
+  <dimension ref="A1:N52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -10355,26 +11683,33 @@
         <f>IF('Profit &amp; Loss'!F4=0,"",'Profit &amp; Loss'!G4/'Profit &amp; Loss'!F4-1)</f>
         <v/>
       </c>
-      <c r="H5" s="24" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="I5" s="24" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="J5" s="24" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="K5" s="24" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="L5" s="24" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="M5" s="24" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="N5" s="24" t="n">
-        <v>0.11</v>
+      <c r="H5" s="79">
+        <f>IF(G44=0,"",H44/G44-1)</f>
+        <v/>
+      </c>
+      <c r="I5" s="79">
+        <f>IF(H44=0,"",I44/H44-1)</f>
+        <v/>
+      </c>
+      <c r="J5" s="79">
+        <f>IF(I44=0,"",J44/I44-1)</f>
+        <v/>
+      </c>
+      <c r="K5" s="79">
+        <f>IF(J44=0,"",K44/J44-1)</f>
+        <v/>
+      </c>
+      <c r="L5" s="79">
+        <f>IF(K44=0,"",L44/K44-1)</f>
+        <v/>
+      </c>
+      <c r="M5" s="79">
+        <f>IF(L44=0,"",M44/L44-1)</f>
+        <v/>
+      </c>
+      <c r="N5" s="79">
+        <f>IF(M44=0,"",N44/M44-1)</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -10407,25 +11742,25 @@
         <f>'Profit &amp; Loss'!G6/'Profit &amp; Loss'!G4</f>
         <v/>
       </c>
-      <c r="H6" s="24" t="n">
+      <c r="H6" s="76" t="n">
         <v>0.41</v>
       </c>
-      <c r="I6" s="24" t="n">
+      <c r="I6" s="76" t="n">
         <v>0.41</v>
       </c>
-      <c r="J6" s="24" t="n">
+      <c r="J6" s="76" t="n">
         <v>0.41</v>
       </c>
-      <c r="K6" s="24" t="n">
+      <c r="K6" s="76" t="n">
         <v>0.41</v>
       </c>
-      <c r="L6" s="24" t="n">
+      <c r="L6" s="76" t="n">
         <v>0.41</v>
       </c>
-      <c r="M6" s="24" t="n">
+      <c r="M6" s="76" t="n">
         <v>0.41</v>
       </c>
-      <c r="N6" s="24" t="n">
+      <c r="N6" s="76" t="n">
         <v>0.41</v>
       </c>
     </row>
@@ -10459,25 +11794,25 @@
         <f>'Profit &amp; Loss'!G7/'Profit &amp; Loss'!G4</f>
         <v/>
       </c>
-      <c r="H7" s="24" t="n">
+      <c r="H7" s="76" t="n">
         <v>0.1</v>
       </c>
-      <c r="I7" s="24" t="n">
+      <c r="I7" s="76" t="n">
         <v>0.1</v>
       </c>
-      <c r="J7" s="24" t="n">
+      <c r="J7" s="76" t="n">
         <v>0.105</v>
       </c>
-      <c r="K7" s="24" t="n">
+      <c r="K7" s="76" t="n">
         <v>0.105</v>
       </c>
-      <c r="L7" s="24" t="n">
+      <c r="L7" s="76" t="n">
         <v>0.11</v>
       </c>
-      <c r="M7" s="24" t="n">
+      <c r="M7" s="76" t="n">
         <v>0.11</v>
       </c>
-      <c r="N7" s="24" t="n">
+      <c r="N7" s="76" t="n">
         <v>0.11</v>
       </c>
     </row>
@@ -10511,25 +11846,25 @@
         <f>'Profit &amp; Loss'!G8/'Profit &amp; Loss'!G4</f>
         <v/>
       </c>
-      <c r="H8" s="24" t="n">
+      <c r="H8" s="76" t="n">
         <v>0.18</v>
       </c>
-      <c r="I8" s="24" t="n">
+      <c r="I8" s="76" t="n">
         <v>0.185</v>
       </c>
-      <c r="J8" s="24" t="n">
+      <c r="J8" s="76" t="n">
         <v>0.185</v>
       </c>
-      <c r="K8" s="24" t="n">
+      <c r="K8" s="76" t="n">
         <v>0.185</v>
       </c>
-      <c r="L8" s="24" t="n">
+      <c r="L8" s="76" t="n">
         <v>0.185</v>
       </c>
-      <c r="M8" s="24" t="n">
+      <c r="M8" s="76" t="n">
         <v>0.185</v>
       </c>
-      <c r="N8" s="24" t="n">
+      <c r="N8" s="76" t="n">
         <v>0.185</v>
       </c>
     </row>
@@ -10563,25 +11898,25 @@
         <f>'Profit &amp; Loss'!G14/'Profit &amp; Loss'!G4</f>
         <v/>
       </c>
-      <c r="H9" s="24" t="n">
+      <c r="H9" s="76" t="n">
         <v>0.015</v>
       </c>
-      <c r="I9" s="24" t="n">
+      <c r="I9" s="76" t="n">
         <v>0.015</v>
       </c>
-      <c r="J9" s="24" t="n">
+      <c r="J9" s="76" t="n">
         <v>0.015</v>
       </c>
-      <c r="K9" s="24" t="n">
+      <c r="K9" s="76" t="n">
         <v>0.015</v>
       </c>
-      <c r="L9" s="24" t="n">
+      <c r="L9" s="76" t="n">
         <v>0.015</v>
       </c>
-      <c r="M9" s="24" t="n">
+      <c r="M9" s="76" t="n">
         <v>0.015</v>
       </c>
-      <c r="N9" s="24" t="n">
+      <c r="N9" s="76" t="n">
         <v>0.015</v>
       </c>
     </row>
@@ -10612,25 +11947,25 @@
         <f>IF('Balance Sheet'!F5=0,"",'Profit &amp; Loss'!G12/'Balance Sheet'!F5)</f>
         <v/>
       </c>
-      <c r="H10" s="24" t="n">
+      <c r="H10" s="76" t="n">
         <v>0.06</v>
       </c>
-      <c r="I10" s="24" t="n">
+      <c r="I10" s="76" t="n">
         <v>0.06</v>
       </c>
-      <c r="J10" s="24" t="n">
+      <c r="J10" s="76" t="n">
         <v>0.06</v>
       </c>
-      <c r="K10" s="24" t="n">
+      <c r="K10" s="76" t="n">
         <v>0.06</v>
       </c>
-      <c r="L10" s="24" t="n">
+      <c r="L10" s="76" t="n">
         <v>0.06</v>
       </c>
-      <c r="M10" s="24" t="n">
+      <c r="M10" s="76" t="n">
         <v>0.06</v>
       </c>
-      <c r="N10" s="24" t="n">
+      <c r="N10" s="76" t="n">
         <v>0.06</v>
       </c>
     </row>
@@ -10710,25 +12045,25 @@
         <f>IF('Profit &amp; Loss'!G18=0,"",'Profit &amp; Loss'!G19/'Profit &amp; Loss'!G18)</f>
         <v/>
       </c>
-      <c r="H12" s="24" t="n">
+      <c r="H12" s="76" t="n">
         <v>0.25</v>
       </c>
-      <c r="I12" s="24" t="n">
+      <c r="I12" s="76" t="n">
         <v>0.25</v>
       </c>
-      <c r="J12" s="24" t="n">
+      <c r="J12" s="76" t="n">
         <v>0.25</v>
       </c>
-      <c r="K12" s="24" t="n">
+      <c r="K12" s="76" t="n">
         <v>0.25</v>
       </c>
-      <c r="L12" s="24" t="n">
+      <c r="L12" s="76" t="n">
         <v>0.25</v>
       </c>
-      <c r="M12" s="24" t="n">
+      <c r="M12" s="76" t="n">
         <v>0.25</v>
       </c>
-      <c r="N12" s="24" t="n">
+      <c r="N12" s="76" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -10744,25 +12079,25 @@
       <c r="E13" s="27" t="inlineStr"/>
       <c r="F13" s="27" t="inlineStr"/>
       <c r="G13" s="27" t="inlineStr"/>
-      <c r="H13" s="24" t="n">
+      <c r="H13" s="76" t="n">
         <v>0.15</v>
       </c>
-      <c r="I13" s="24" t="n">
+      <c r="I13" s="76" t="n">
         <v>0.15</v>
       </c>
-      <c r="J13" s="24" t="n">
+      <c r="J13" s="76" t="n">
         <v>0.15</v>
       </c>
-      <c r="K13" s="24" t="n">
+      <c r="K13" s="76" t="n">
         <v>0.15</v>
       </c>
-      <c r="L13" s="24" t="n">
+      <c r="L13" s="76" t="n">
         <v>0.15</v>
       </c>
-      <c r="M13" s="24" t="n">
+      <c r="M13" s="76" t="n">
         <v>0.15</v>
       </c>
-      <c r="N13" s="24" t="n">
+      <c r="N13" s="76" t="n">
         <v>0.15</v>
       </c>
     </row>
@@ -10952,25 +12287,25 @@
         <f>'Balance Sheet'!G12/'Profit &amp; Loss'!G4</f>
         <v/>
       </c>
-      <c r="H17" s="24" t="n">
+      <c r="H17" s="76" t="n">
         <v>0.06</v>
       </c>
-      <c r="I17" s="24" t="n">
+      <c r="I17" s="76" t="n">
         <v>0.06</v>
       </c>
-      <c r="J17" s="24" t="n">
+      <c r="J17" s="76" t="n">
         <v>0.06</v>
       </c>
-      <c r="K17" s="24" t="n">
+      <c r="K17" s="76" t="n">
         <v>0.06</v>
       </c>
-      <c r="L17" s="24" t="n">
+      <c r="L17" s="76" t="n">
         <v>0.06</v>
       </c>
-      <c r="M17" s="24" t="n">
+      <c r="M17" s="76" t="n">
         <v>0.06</v>
       </c>
-      <c r="N17" s="24" t="n">
+      <c r="N17" s="76" t="n">
         <v>0.06</v>
       </c>
     </row>
@@ -11004,25 +12339,25 @@
         <f>'Balance Sheet'!G22/'Profit &amp; Loss'!G4</f>
         <v/>
       </c>
-      <c r="H18" s="24" t="n">
+      <c r="H18" s="76" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="I18" s="24" t="n">
+      <c r="I18" s="76" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="J18" s="24" t="n">
+      <c r="J18" s="76" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="K18" s="24" t="n">
+      <c r="K18" s="76" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="L18" s="24" t="n">
+      <c r="L18" s="76" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="M18" s="24" t="n">
+      <c r="M18" s="76" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="N18" s="24" t="n">
+      <c r="N18" s="76" t="n">
         <v>0.07000000000000001</v>
       </c>
     </row>
@@ -11105,25 +12440,25 @@
         <f>IF('Balance Sheet'!F18=0,"",'Profit &amp; Loss'!G15/(('Balance Sheet'!F18+'Balance Sheet'!G18)/2))</f>
         <v/>
       </c>
-      <c r="H20" s="24" t="n">
+      <c r="H20" s="76" t="n">
         <v>0.075</v>
       </c>
-      <c r="I20" s="24" t="n">
+      <c r="I20" s="76" t="n">
         <v>0.075</v>
       </c>
-      <c r="J20" s="24" t="n">
+      <c r="J20" s="76" t="n">
         <v>0.075</v>
       </c>
-      <c r="K20" s="24" t="n">
+      <c r="K20" s="76" t="n">
         <v>0.075</v>
       </c>
-      <c r="L20" s="24" t="n">
+      <c r="L20" s="76" t="n">
         <v>0.075</v>
       </c>
-      <c r="M20" s="24" t="n">
+      <c r="M20" s="76" t="n">
         <v>0.075</v>
       </c>
-      <c r="N20" s="24" t="n">
+      <c r="N20" s="76" t="n">
         <v>0.075</v>
       </c>
     </row>
@@ -11267,8 +12602,425 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="18" t="inlineStr">
+        <is>
+          <t>Revenue build by business segment (Rs Cr) - estimated mix</t>
+        </is>
+      </c>
+      <c r="B40" s="19" t="n"/>
+      <c r="C40" s="19" t="n"/>
+      <c r="D40" s="19" t="n"/>
+      <c r="E40" s="19" t="n"/>
+      <c r="F40" s="19" t="n"/>
+      <c r="G40" s="19" t="n"/>
+      <c r="H40" s="19" t="n"/>
+      <c r="I40" s="19" t="n"/>
+      <c r="J40" s="19" t="n"/>
+      <c r="K40" s="19" t="n"/>
+      <c r="L40" s="19" t="n"/>
+      <c r="M40" s="19" t="n"/>
+      <c r="N40" s="19" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>HPP, Refrigerants &amp; Inorganic fluorides</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="n">
+        <v>601.49</v>
+      </c>
+      <c r="C41" s="12" t="n">
+        <v>726.6799999999999</v>
+      </c>
+      <c r="D41" s="12" t="n">
+        <v>1017.93</v>
+      </c>
+      <c r="E41" s="12" t="n">
+        <v>1073.81</v>
+      </c>
+      <c r="F41" s="12" t="n">
+        <v>1127.7</v>
+      </c>
+      <c r="G41" s="12" t="n">
+        <v>1524.44</v>
+      </c>
+      <c r="H41" s="13">
+        <f>G41*(1+H47)</f>
+        <v/>
+      </c>
+      <c r="I41" s="13">
+        <f>H41*(1+I47)</f>
+        <v/>
+      </c>
+      <c r="J41" s="13">
+        <f>I41*(1+J47)</f>
+        <v/>
+      </c>
+      <c r="K41" s="13">
+        <f>J41*(1+K47)</f>
+        <v/>
+      </c>
+      <c r="L41" s="13">
+        <f>K41*(1+L47)</f>
+        <v/>
+      </c>
+      <c r="M41" s="13">
+        <f>L41*(1+M47)</f>
+        <v/>
+      </c>
+      <c r="N41" s="13">
+        <f>M41*(1+N47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>Specialty Chemicals</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="n">
+        <v>459.96</v>
+      </c>
+      <c r="C42" s="12" t="n">
+        <v>566.8099999999999</v>
+      </c>
+      <c r="D42" s="12" t="n">
+        <v>789.41</v>
+      </c>
+      <c r="E42" s="12" t="n">
+        <v>764.05</v>
+      </c>
+      <c r="F42" s="12" t="n">
+        <v>869.27</v>
+      </c>
+      <c r="G42" s="12" t="n">
+        <v>1325.6</v>
+      </c>
+      <c r="H42" s="13">
+        <f>G42*(1+H48)</f>
+        <v/>
+      </c>
+      <c r="I42" s="13">
+        <f>H42*(1+I48)</f>
+        <v/>
+      </c>
+      <c r="J42" s="13">
+        <f>I42*(1+J48)</f>
+        <v/>
+      </c>
+      <c r="K42" s="13">
+        <f>J42*(1+K48)</f>
+        <v/>
+      </c>
+      <c r="L42" s="13">
+        <f>K42*(1+L48)</f>
+        <v/>
+      </c>
+      <c r="M42" s="13">
+        <f>L42*(1+M48)</f>
+        <v/>
+      </c>
+      <c r="N42" s="13">
+        <f>M42*(1+N48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t>CDMO / CRAMS</t>
+        </is>
+      </c>
+      <c r="B43" s="13">
+        <f>'Profit &amp; Loss'!B4-B41-B42</f>
+        <v/>
+      </c>
+      <c r="C43" s="13">
+        <f>'Profit &amp; Loss'!C4-C41-C42</f>
+        <v/>
+      </c>
+      <c r="D43" s="13">
+        <f>'Profit &amp; Loss'!D4-D41-D42</f>
+        <v/>
+      </c>
+      <c r="E43" s="13">
+        <f>'Profit &amp; Loss'!E4-E41-E42</f>
+        <v/>
+      </c>
+      <c r="F43" s="13">
+        <f>'Profit &amp; Loss'!F4-F41-F42</f>
+        <v/>
+      </c>
+      <c r="G43" s="13">
+        <f>'Profit &amp; Loss'!G4-G41-G42</f>
+        <v/>
+      </c>
+      <c r="H43" s="13">
+        <f>G43*(1+H49)</f>
+        <v/>
+      </c>
+      <c r="I43" s="13">
+        <f>H43*(1+I49)</f>
+        <v/>
+      </c>
+      <c r="J43" s="13">
+        <f>I43*(1+J49)</f>
+        <v/>
+      </c>
+      <c r="K43" s="13">
+        <f>J43*(1+K49)</f>
+        <v/>
+      </c>
+      <c r="L43" s="13">
+        <f>K43*(1+L49)</f>
+        <v/>
+      </c>
+      <c r="M43" s="13">
+        <f>L43*(1+M49)</f>
+        <v/>
+      </c>
+      <c r="N43" s="13">
+        <f>M43*(1+N49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>Total revenue</t>
+        </is>
+      </c>
+      <c r="B44" s="14">
+        <f>SUM(B41:B43)</f>
+        <v/>
+      </c>
+      <c r="C44" s="14">
+        <f>SUM(C41:C43)</f>
+        <v/>
+      </c>
+      <c r="D44" s="14">
+        <f>SUM(D41:D43)</f>
+        <v/>
+      </c>
+      <c r="E44" s="14">
+        <f>SUM(E41:E43)</f>
+        <v/>
+      </c>
+      <c r="F44" s="14">
+        <f>SUM(F41:F43)</f>
+        <v/>
+      </c>
+      <c r="G44" s="14">
+        <f>SUM(G41:G43)</f>
+        <v/>
+      </c>
+      <c r="H44" s="14">
+        <f>SUM(H41:H43)</f>
+        <v/>
+      </c>
+      <c r="I44" s="14">
+        <f>SUM(I41:I43)</f>
+        <v/>
+      </c>
+      <c r="J44" s="14">
+        <f>SUM(J41:J43)</f>
+        <v/>
+      </c>
+      <c r="K44" s="14">
+        <f>SUM(K41:K43)</f>
+        <v/>
+      </c>
+      <c r="L44" s="14">
+        <f>SUM(L41:L43)</f>
+        <v/>
+      </c>
+      <c r="M44" s="14">
+        <f>SUM(M41:M43)</f>
+        <v/>
+      </c>
+      <c r="N44" s="14">
+        <f>SUM(N41:N43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="18" t="inlineStr">
+        <is>
+          <t>Segment growth assumptions (%)</t>
+        </is>
+      </c>
+      <c r="B46" s="19" t="n"/>
+      <c r="C46" s="19" t="n"/>
+      <c r="D46" s="19" t="n"/>
+      <c r="E46" s="19" t="n"/>
+      <c r="F46" s="19" t="n"/>
+      <c r="G46" s="19" t="n"/>
+      <c r="H46" s="19" t="n"/>
+      <c r="I46" s="19" t="n"/>
+      <c r="J46" s="19" t="n"/>
+      <c r="K46" s="19" t="n"/>
+      <c r="L46" s="19" t="n"/>
+      <c r="M46" s="19" t="n"/>
+      <c r="N46" s="19" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>HPP / Refrigerants growth</t>
+        </is>
+      </c>
+      <c r="C47" s="10">
+        <f>IF(B41=0,"",C41/B41-1)</f>
+        <v/>
+      </c>
+      <c r="D47" s="10">
+        <f>IF(C41=0,"",D41/C41-1)</f>
+        <v/>
+      </c>
+      <c r="E47" s="10">
+        <f>IF(D41=0,"",E41/D41-1)</f>
+        <v/>
+      </c>
+      <c r="F47" s="10">
+        <f>IF(E41=0,"",F41/E41-1)</f>
+        <v/>
+      </c>
+      <c r="G47" s="10">
+        <f>IF(F41=0,"",G41/F41-1)</f>
+        <v/>
+      </c>
+      <c r="H47" s="76" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="I47" s="76" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="J47" s="76" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="K47" s="76" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="L47" s="76" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M47" s="76" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N47" s="76" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="inlineStr">
+        <is>
+          <t>Specialty Chemicals growth</t>
+        </is>
+      </c>
+      <c r="C48" s="10">
+        <f>IF(B42=0,"",C42/B42-1)</f>
+        <v/>
+      </c>
+      <c r="D48" s="10">
+        <f>IF(C42=0,"",D42/C42-1)</f>
+        <v/>
+      </c>
+      <c r="E48" s="10">
+        <f>IF(D42=0,"",E42/D42-1)</f>
+        <v/>
+      </c>
+      <c r="F48" s="10">
+        <f>IF(E42=0,"",F42/E42-1)</f>
+        <v/>
+      </c>
+      <c r="G48" s="10">
+        <f>IF(F42=0,"",G42/F42-1)</f>
+        <v/>
+      </c>
+      <c r="H48" s="76" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="I48" s="76" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="J48" s="76" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="K48" s="76" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="L48" s="76" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="M48" s="76" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="N48" s="76" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
+        <is>
+          <t>CDMO / CRAMS growth</t>
+        </is>
+      </c>
+      <c r="C49" s="10">
+        <f>IF(B43=0,"",C43/B43-1)</f>
+        <v/>
+      </c>
+      <c r="D49" s="10">
+        <f>IF(C43=0,"",D43/C43-1)</f>
+        <v/>
+      </c>
+      <c r="E49" s="10">
+        <f>IF(D43=0,"",E43/D43-1)</f>
+        <v/>
+      </c>
+      <c r="F49" s="10">
+        <f>IF(E43=0,"",F43/E43-1)</f>
+        <v/>
+      </c>
+      <c r="G49" s="10">
+        <f>IF(F43=0,"",G43/F43-1)</f>
+        <v/>
+      </c>
+      <c r="H49" s="76" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I49" s="76" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="J49" s="76" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K49" s="76" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="L49" s="76" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M49" s="76" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="N49" s="76" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="50" ht="44" customHeight="1">
+      <c r="A50" s="53" t="inlineStr">
+        <is>
+          <t>Note: Segment split is an analyst estimate anchored to disclosed quarterly mix (e.g. Q3FY26: HPP Rs412 Cr, Specialty Rs354 Cr, CDMO Rs127 Cr) and management growth commentary; CDMO modelled as the fastest grower on cGMP-4 ramp. Total revenue feeds the P&amp;L.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51"/>
+    <row r="52"/>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="B31:N31"/>
     <mergeCell ref="B27:N27"/>
     <mergeCell ref="B32:N32"/>
@@ -11278,6 +13030,7 @@
     <mergeCell ref="B33:N33"/>
     <mergeCell ref="B25:N25"/>
     <mergeCell ref="B24:N24"/>
+    <mergeCell ref="A50:N52"/>
     <mergeCell ref="B28:N28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add live scenario toggle, computed regression beta
- Live Bull/Base/Bear selector (Assumptions!B55, dropdown) that flexes
  segment revenue growth, EBITDA margin, WACC, terminal growth and exit
  multiple across the whole model; balance sheet balances under all three.
- Beta now a computed regression: 0.91 (3yr) / 0.83 (5yr) monthly
  NAVINFLUOR vs Nifty 50, replacing the published-beta placeholder.
- DCF WACC/terminal growth/exit multiple are scenario-driven; CAPM WACC
  retained as a reference.
</commit_message>
<xml_diff>
--- a/Navin Fluorine International - Financial Model.xlsx
+++ b/Navin Fluorine International - Financial Model.xlsx
@@ -188,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -297,7 +297,7 @@
     <xf numFmtId="10" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="12" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -421,6 +421,33 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="12" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -3996,11 +4023,11 @@
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>Raw levered beta (2-yr monthly vs index; published)</t>
+          <t>Raw levered beta - 3yr monthly regression vs Nifty 50 (computed)</t>
         </is>
       </c>
       <c r="B5" s="45" t="n">
-        <v>0.89</v>
+        <v>0.912</v>
       </c>
     </row>
     <row r="6">
@@ -4017,8 +4044,11 @@
     <row r="7">
       <c r="A7" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (Source: BusinessToday / exchange data, Jun-2026)</t>
-        </is>
+          <t>Raw levered beta - 5yr monthly regression (reference)</t>
+        </is>
+      </c>
+      <c r="B7" s="88" t="n">
+        <v>0.828</v>
       </c>
     </row>
     <row r="9">
@@ -4230,7 +4260,7 @@
     <row r="24" ht="48" customHeight="1">
       <c r="A24" s="53" t="inlineStr">
         <is>
-          <t>Note: Navin operates near net-cash; peer betas reflect listed Indian specialty-chemical comparables. A regression beta would be computed from 24-36 monthly returns of NAVINFLUOR vs the Nifty 500; the published adjusted beta (~0.89) is used as the regression proxy.</t>
+          <t>Note: Raw beta computed by regressing 36 monthly returns of NAVINFLUOR (NSE) on the Nifty 50 (beta = Cov/Var) = 0.91 (3yr); 5yr = 0.83; consistent with published ~0.89. Blume-adjusted and bottom-up (peer) approaches are averaged for the selected beta used in the cost of equity.</t>
         </is>
       </c>
     </row>
@@ -6317,13 +6347,13 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>WACC</t>
-        </is>
-      </c>
-      <c r="B16" s="38">
-        <f>B14*B8+B15*B11</f>
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>WACC  (scenario-driven)</t>
+        </is>
+      </c>
+      <c r="B16" s="80">
+        <f>Assumptions!B59</f>
         <v/>
       </c>
     </row>
@@ -6333,8 +6363,20 @@
           <t>Terminal growth rate (g)</t>
         </is>
       </c>
-      <c r="B17" s="76" t="n">
-        <v>0.055</v>
+      <c r="B17" s="81">
+        <f>Assumptions!B60</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   CAPM WACC (reference) = We x Ke + Wd x Kd(1-t)</t>
+        </is>
+      </c>
+      <c r="B18" s="10">
+        <f>B14*B8+B15*B11</f>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -7017,8 +7059,9 @@
           <t>Exit EV/EBITDA multiple (x)</t>
         </is>
       </c>
-      <c r="B70" s="45" t="n">
-        <v>18</v>
+      <c r="B70" s="82">
+        <f>Assumptions!B61</f>
+        <v/>
       </c>
     </row>
     <row r="71">
@@ -8801,31 +8844,31 @@
         <v>542</v>
       </c>
       <c r="H8" s="13">
-        <f>H4*Assumptions!H8</f>
+        <f>H4*(Assumptions!H8-Assumptions!$B$58)</f>
         <v/>
       </c>
       <c r="I8" s="13">
-        <f>I4*Assumptions!I8</f>
+        <f>I4*(Assumptions!I8-Assumptions!$B$58)</f>
         <v/>
       </c>
       <c r="J8" s="13">
-        <f>J4*Assumptions!J8</f>
+        <f>J4*(Assumptions!J8-Assumptions!$B$58)</f>
         <v/>
       </c>
       <c r="K8" s="13">
-        <f>K4*Assumptions!K8</f>
+        <f>K4*(Assumptions!K8-Assumptions!$B$58)</f>
         <v/>
       </c>
       <c r="L8" s="13">
-        <f>L4*Assumptions!L8</f>
+        <f>L4*(Assumptions!L8-Assumptions!$B$58)</f>
         <v/>
       </c>
       <c r="M8" s="13">
-        <f>M4*Assumptions!M8</f>
+        <f>M4*(Assumptions!M8-Assumptions!$B$58)</f>
         <v/>
       </c>
       <c r="N8" s="13">
-        <f>N4*Assumptions!N8</f>
+        <f>N4*(Assumptions!N8-Assumptions!$B$58)</f>
         <v/>
       </c>
     </row>
@@ -11538,7 +11581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N52"/>
+  <dimension ref="A1:N61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -12647,31 +12690,31 @@
         <v>1524.44</v>
       </c>
       <c r="H41" s="13">
-        <f>G41*(1+H47)</f>
+        <f>G41*(1+H47+$B$57)</f>
         <v/>
       </c>
       <c r="I41" s="13">
-        <f>H41*(1+I47)</f>
+        <f>H41*(1+I47+$B$57)</f>
         <v/>
       </c>
       <c r="J41" s="13">
-        <f>I41*(1+J47)</f>
+        <f>I41*(1+J47+$B$57)</f>
         <v/>
       </c>
       <c r="K41" s="13">
-        <f>J41*(1+K47)</f>
+        <f>J41*(1+K47+$B$57)</f>
         <v/>
       </c>
       <c r="L41" s="13">
-        <f>K41*(1+L47)</f>
+        <f>K41*(1+L47+$B$57)</f>
         <v/>
       </c>
       <c r="M41" s="13">
-        <f>L41*(1+M47)</f>
+        <f>L41*(1+M47+$B$57)</f>
         <v/>
       </c>
       <c r="N41" s="13">
-        <f>M41*(1+N47)</f>
+        <f>M41*(1+N47+$B$57)</f>
         <v/>
       </c>
     </row>
@@ -12700,31 +12743,31 @@
         <v>1325.6</v>
       </c>
       <c r="H42" s="13">
-        <f>G42*(1+H48)</f>
+        <f>G42*(1+H48+$B$57)</f>
         <v/>
       </c>
       <c r="I42" s="13">
-        <f>H42*(1+I48)</f>
+        <f>H42*(1+I48+$B$57)</f>
         <v/>
       </c>
       <c r="J42" s="13">
-        <f>I42*(1+J48)</f>
+        <f>I42*(1+J48+$B$57)</f>
         <v/>
       </c>
       <c r="K42" s="13">
-        <f>J42*(1+K48)</f>
+        <f>J42*(1+K48+$B$57)</f>
         <v/>
       </c>
       <c r="L42" s="13">
-        <f>K42*(1+L48)</f>
+        <f>K42*(1+L48+$B$57)</f>
         <v/>
       </c>
       <c r="M42" s="13">
-        <f>L42*(1+M48)</f>
+        <f>L42*(1+M48+$B$57)</f>
         <v/>
       </c>
       <c r="N42" s="13">
-        <f>M42*(1+N48)</f>
+        <f>M42*(1+N48+$B$57)</f>
         <v/>
       </c>
     </row>
@@ -12759,31 +12802,31 @@
         <v/>
       </c>
       <c r="H43" s="13">
-        <f>G43*(1+H49)</f>
+        <f>G43*(1+H49+$B$57)</f>
         <v/>
       </c>
       <c r="I43" s="13">
-        <f>H43*(1+I49)</f>
+        <f>H43*(1+I49+$B$57)</f>
         <v/>
       </c>
       <c r="J43" s="13">
-        <f>I43*(1+J49)</f>
+        <f>I43*(1+J49+$B$57)</f>
         <v/>
       </c>
       <c r="K43" s="13">
-        <f>J43*(1+K49)</f>
+        <f>J43*(1+K49+$B$57)</f>
         <v/>
       </c>
       <c r="L43" s="13">
-        <f>K43*(1+L49)</f>
+        <f>K43*(1+L49+$B$57)</f>
         <v/>
       </c>
       <c r="M43" s="13">
-        <f>L43*(1+M49)</f>
+        <f>L43*(1+M49+$B$57)</f>
         <v/>
       </c>
       <c r="N43" s="13">
-        <f>M43*(1+N49)</f>
+        <f>M43*(1+N49+$B$57)</f>
         <v/>
       </c>
     </row>
@@ -13019,6 +13062,163 @@
     </row>
     <row r="51"/>
     <row r="52"/>
+    <row r="54">
+      <c r="A54" s="18" t="inlineStr">
+        <is>
+          <t>Scenario control  (switch drives the whole model &amp; valuation)</t>
+        </is>
+      </c>
+      <c r="B54" s="19" t="n"/>
+      <c r="C54" s="19" t="n"/>
+      <c r="D54" s="19" t="n"/>
+      <c r="E54" s="19" t="n"/>
+      <c r="F54" s="19" t="n"/>
+      <c r="G54" s="19" t="n"/>
+      <c r="H54" s="19" t="n"/>
+      <c r="I54" s="19" t="n"/>
+      <c r="J54" s="19" t="n"/>
+      <c r="K54" s="19" t="n"/>
+      <c r="L54" s="19" t="n"/>
+      <c r="M54" s="19" t="n"/>
+      <c r="N54" s="19" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>Scenario selector  (1 = Bull, 2 = Base, 3 = Bear)</t>
+        </is>
+      </c>
+      <c r="B55" s="83" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Driver</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="11" t="inlineStr">
+        <is>
+          <t>Revenue growth delta (pp on each segment)</t>
+        </is>
+      </c>
+      <c r="B57" s="84">
+        <f>CHOOSE($B$55,C57,D57,E57)</f>
+        <v/>
+      </c>
+      <c r="C57" s="85" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D57" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" s="85" t="n">
+        <v>-0.03</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t>EBITDA margin delta (pp)</t>
+        </is>
+      </c>
+      <c r="B58" s="84">
+        <f>CHOOSE($B$55,C58,D58,E58)</f>
+        <v/>
+      </c>
+      <c r="C58" s="85" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="D58" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" s="85" t="n">
+        <v>-0.02</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="11" t="inlineStr">
+        <is>
+          <t>WACC</t>
+        </is>
+      </c>
+      <c r="B59" s="86">
+        <f>CHOOSE($B$55,C59,D59,E59)</f>
+        <v/>
+      </c>
+      <c r="C59" s="87" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="D59" s="87" t="n">
+        <v>0.117</v>
+      </c>
+      <c r="E59" s="87" t="n">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>Terminal growth rate</t>
+        </is>
+      </c>
+      <c r="B60" s="86">
+        <f>CHOOSE($B$55,C60,D60,E60)</f>
+        <v/>
+      </c>
+      <c r="C60" s="87" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D60" s="87" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="E60" s="87" t="n">
+        <v>0.045</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="11" t="inlineStr">
+        <is>
+          <t>Exit EV/EBITDA multiple (x)</t>
+        </is>
+      </c>
+      <c r="B61" s="52">
+        <f>CHOOSE($B$55,C61,D61,E61)</f>
+        <v/>
+      </c>
+      <c r="C61" s="73" t="n">
+        <v>22</v>
+      </c>
+      <c r="D61" s="73" t="n">
+        <v>18</v>
+      </c>
+      <c r="E61" s="73" t="n">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="B31:N31"/>
@@ -13033,6 +13233,11 @@
     <mergeCell ref="A50:N52"/>
     <mergeCell ref="B28:N28"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"1,2,3"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Embed industry & company insight into the model narrative
- Enriched Summary investment thesis with structural drivers: India
  fluorochemicals/specialty-gases ~16-18% CAGR, Kigali HFC phase-down /
  R-32 shift, CDMO cGMP-4 + oncology pipeline, ~Rs1,400 Cr capex incl
  AI-cooling/EV-fluorine optionality, China+1 scarcity, and key risks.
- Added an 'Industry & company context' section in Notes to Accounts
  mapping each insight to the model driver it informs, with sources
  (kept within existing sheets per the brief - no separate insights sheet).
</commit_message>
<xml_diff>
--- a/Navin Fluorine International - Financial Model.xlsx
+++ b/Navin Fluorine International - Financial Model.xlsx
@@ -188,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -449,6 +449,13 @@
     </xf>
     <xf numFmtId="167" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -979,7 +986,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>39</row>
+      <row>42</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="2700000"/>
@@ -1001,7 +1008,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>55</row>
+      <row>58</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="2700000"/>
@@ -1365,7 +1372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N37"/>
+  <dimension ref="A1:N38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2236,49 +2243,57 @@
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="31" t="inlineStr">
         <is>
-          <t>+  Structural growth: ~15% revenue CAGR FY26-33 driven by HPP (R-32/HFOs), CDMO/CRAMS ramp (cGMP-4, MPP), agro-specialties and capacity expansion at Dahej &amp; Surat.</t>
+          <t>+  Structural demand: India fluorochemicals / specialty-gases market is projected to grow ~16-18% CAGR (FY24-29), pulled by pharma, agro, electronics &amp; semiconductors, autos and emerging EV-battery fluorine (LiPF6) and data-centre / 'AI cooling' fluids - underpins our ~15% revenue CAGR and CDMO being the fastest segment.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="31" t="inlineStr">
         <is>
-          <t>+  Premium franchise: scarcity value as an integrated fluorination + AHF player; high-value specialty mix lifted FY26 EBITDA margin to 32.6% and PAT 2.3x YoY.</t>
+          <t>+  Refrigerant transition: the Kigali HFC phase-down (India freezes consumption ~2028, cuts from 2032) is shifting demand toward low-GWP R-32 / HFOs where Navin has added capacity - supports HPP pricing and volumes through the transition.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="31" t="inlineStr">
         <is>
-          <t>+  Strong balance sheet: Rs750 Cr QIP (Jul-2025) funds the capex cycle; company operates near net-cash with comfortable interest cover.</t>
+          <t>+  Premiumisation &amp; CDMO: deliberate shift to high-margin custom manufacturing; cGMP-4 commercial supplies have begun with a balanced oncology / late-stage pipeline (CDMO +61% YoY in Q4FY26) - drives the margin (FY26 32.6% vs the 25-30% long-term target) and the mix.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="31" t="inlineStr">
         <is>
-          <t>-  Valuation: trades at ~58x trailing P/E and ~9.8x book; our DCF (WACC ~11.7%, g 5.5%) and peer-relative valuation both sit below the current price.</t>
+          <t>+  Capex &amp; balance sheet: a ~Rs1,400 Cr multi-year programme (Dahej MPP / agro-specialty, Surat HFC / R-32, cGMP-4) funded by the Rs750 Cr QIP (Jul-2025); near net-cash - reflected in our capex and deleveraging path.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="31" t="inlineStr">
         <is>
-          <t>-  Risks: customer concentration in CDMO, raw-material/fluorspar pricing, refrigerant cycle, forex, and execution on large projects.</t>
+          <t>+  China+1 / scarcity: integrated fluorination with captive AHF is a high-barrier, scarce capability that benefits from global supply-chain diversification away from China.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="31" t="inlineStr">
         <is>
-          <t>&gt;  Net view: Rating reflects rich valuation, not business quality. Fair value range Rs 4,000-5,500; accumulate on meaningful corrections.</t>
+          <t>-  Valuation &amp; risks: ~58x trailing P/E and ~9.8x book; CDMO customer concentration, fluorspar / raw-material (China-linked) and forex exposure, agchem pricing pressure and refrigerant cyclicality (captured in the Bear scenario).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="31" t="inlineStr">
+        <is>
+          <t>&gt;  Net view: a high-quality structural compounder, but a rich valuation drives our disciplined Reduce/Neutral stance - base fair value Rs ~4,000-5,500, bull case ~Rs7,600. Accumulate on meaningful corrections.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A34:N34"/>
     <mergeCell ref="A35:N35"/>
+    <mergeCell ref="A38:N38"/>
     <mergeCell ref="A5:N7"/>
     <mergeCell ref="A33:N33"/>
     <mergeCell ref="A37:N37"/>
@@ -4280,7 +4295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N37"/>
+  <dimension ref="A1:N48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5091,12 +5106,110 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="89" t="inlineStr">
+        <is>
+          <t>Industry &amp; company context - the insight behind the assumptions</t>
+        </is>
+      </c>
+      <c r="B42" s="19" t="n"/>
+      <c r="C42" s="19" t="n"/>
+      <c r="D42" s="19" t="n"/>
+      <c r="E42" s="19" t="n"/>
+      <c r="F42" s="19" t="n"/>
+      <c r="G42" s="19" t="n"/>
+      <c r="H42" s="19" t="n"/>
+      <c r="I42" s="19" t="n"/>
+      <c r="J42" s="19" t="n"/>
+      <c r="K42" s="19" t="n"/>
+      <c r="L42" s="19" t="n"/>
+      <c r="M42" s="19" t="n"/>
+      <c r="N42" s="19" t="n"/>
+    </row>
+    <row r="43" ht="60" customHeight="1">
+      <c r="A43" s="90" t="inlineStr">
+        <is>
+          <t>Market &amp; growth</t>
+        </is>
+      </c>
+      <c r="B43" s="91" t="inlineStr">
+        <is>
+          <t>India's fluorochemicals / specialty-gases market is estimated to grow ~16-18% CAGR over FY24-29 (fluorochemicals ~10% CAGR off a ~USD0.6bn-2022 base), driven by pharma, agrochemicals, electronics &amp; semiconductors, autos, and emerging EV-battery fluorine (LiPF6). MODEL LINK: supports the ~15% FY26-33 revenue CAGR and the segment build (CDMO fastest). Source: industry research (MarkNtel; Livemint citing 16-18% CAGR).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="60" customHeight="1">
+      <c r="A44" s="90" t="inlineStr">
+        <is>
+          <t>Refrigerant / HFC transition</t>
+        </is>
+      </c>
+      <c r="B44" s="91" t="inlineStr">
+        <is>
+          <t>Under the Kigali Amendment, India freezes HFC consumption around 2028 and phases it down from 2032 (10%) to 2047 (85%), accelerating the shift to low-GWP R-32 and HFOs. The global HFC market (~USD24bn, 2026) is still growing ~4% with R-32 volumes rising on auto/room AC. MODEL LINK: underpins HPP/refrigerant volume and pricing as Navin commissions R-32/HFC capacity at Surat. Source: NextIAS; MarkWide Research.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="60" customHeight="1">
+      <c r="A45" s="90" t="inlineStr">
+        <is>
+          <t>CDMO / pharma outsourcing</t>
+        </is>
+      </c>
+      <c r="B45" s="91" t="inlineStr">
+        <is>
+          <t>cGMP-4 commercial supplies have begun; a balanced early- and late-stage pipeline (incl. oncology) and pharma's China+1 outsourcing drove CDMO revenue +61% YoY in Q4FY26. MODEL LINK: CDMO modelled as the fastest-growing segment (25-30% near term). Source: company results / earnings calls (Quartr).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="60" customHeight="1">
+      <c r="A46" s="90" t="inlineStr">
+        <is>
+          <t>Margin trajectory</t>
+        </is>
+      </c>
+      <c r="B46" s="91" t="inlineStr">
+        <is>
+          <t>Management's long-term EBITDA-margin target is 25-30%; FY26 ran at ~32.6% (Q3FY26 ~34.5%) on a richer custom-manufacturing mix, better realisation and operating leverage. MODEL LINK: forecast EBITDA margin held ~30% (normalising from the FY26 peak, above the old guidance). Source: earnings calls; Indian Express.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="60" customHeight="1">
+      <c r="A47" s="90" t="inlineStr">
+        <is>
+          <t>Capex &amp; optionality</t>
+        </is>
+      </c>
+      <c r="B47" s="91" t="inlineStr">
+        <is>
+          <t>A ~Rs1,400 Cr multi-year programme spans Dahej MPP/agro-specialty (~Rs540 Cr commissioned), Surat HFC/R-32, and cGMP-4 CDMO, with new optionality in oncology CDMO and data-centre/'AI cooling' immersion fluids; funded by the Rs750 Cr QIP. MODEL LINK: capex schedule and the deleveraging/cash-sweep path; AI-cooling/EV-fluorine upside is NOT in the base case (captured in Bull). Source: Indian Express; investor presentations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="60" customHeight="1">
+      <c r="A48" s="90" t="inlineStr">
+        <is>
+          <t>Key risks</t>
+        </is>
+      </c>
+      <c r="B48" s="91" t="inlineStr">
+        <is>
+          <t>CDMO customer concentration; fluorspar / raw-material dependence on China; forex (export-heavy); agrochemical pricing pressure; and refrigerant-pricing cyclicality. MODEL LINK: stressed in the Bear scenario (lower growth &amp; margin, higher WACC). Source: management commentary; industry.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="11">
+    <mergeCell ref="B46:N46"/>
+    <mergeCell ref="B45:N45"/>
     <mergeCell ref="A34:N34"/>
     <mergeCell ref="A35:N35"/>
+    <mergeCell ref="B43:N43"/>
+    <mergeCell ref="B44:N44"/>
     <mergeCell ref="A33:N33"/>
+    <mergeCell ref="B48:N48"/>
     <mergeCell ref="A37:N37"/>
+    <mergeCell ref="B47:N47"/>
     <mergeCell ref="A36:N36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 3-stage DCF to FY2040 and surface scenarios on Summary
- Extended DCF horizon to FY2040 via an explicit Stage-2 fade (FY34-40),
  reducing terminal value from ~78% to ~54% of EV; DCF intrinsic now
  blends Gordon, exit-multiple and 3-stage methods.
- Added a visible Scenario fair-value summary (Bull/Base/Bear + DCF
  3-stage) on the Summary sheet, with a pointer to the live toggle at
  Assumptions!B55.
</commit_message>
<xml_diff>
--- a/Navin Fluorine International - Financial Model.xlsx
+++ b/Navin Fluorine International - Financial Model.xlsx
@@ -188,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -456,6 +456,9 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1450,6 +1453,14 @@
       <c r="D8" s="19" t="n"/>
       <c r="E8" s="19" t="n"/>
       <c r="F8" s="19" t="n"/>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Scenario fair value (Rs/share)</t>
+        </is>
+      </c>
+      <c r="H8" s="19" t="n"/>
+      <c r="I8" s="19" t="n"/>
+      <c r="J8" s="19" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
@@ -1468,6 +1479,15 @@
       <c r="E9" s="60" t="n">
         <v>39032</v>
       </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="J9" s="56">
+        <f>'Valuation Summary'!C77</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
@@ -1487,6 +1507,15 @@
       <c r="E10" s="61" t="n">
         <v>2</v>
       </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="J10" s="56">
+        <f>'Valuation Summary'!C78</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
@@ -1507,6 +1536,15 @@
       <c r="E11" s="59" t="n">
         <v>775</v>
       </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="J11" s="56">
+        <f>'Valuation Summary'!C79</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
@@ -1526,6 +1564,15 @@
       <c r="E12" s="64" t="n">
         <v>9.800000000000001</v>
       </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>DCF 3-stage (to FY2040)</t>
+        </is>
+      </c>
+      <c r="J12" s="56">
+        <f>DCF!B94</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
@@ -1545,6 +1592,15 @@
       <c r="E13" s="65" t="n">
         <v>0.002</v>
       </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>Blended target</t>
+        </is>
+      </c>
+      <c r="J13" s="74">
+        <f>'Valuation Summary'!D35</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
@@ -1562,6 +1618,11 @@
       </c>
       <c r="E14" s="65" t="n">
         <v>0.068</v>
+      </c>
+      <c r="G14" s="47" t="inlineStr">
+        <is>
+          <t>Live toggle: Assumptions!B55 (1=Bull,2=Base,3=Bear)</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -6288,7 +6349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N77"/>
+  <dimension ref="A1:N96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -7246,12 +7307,319 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>DCF value (avg of Gordon-growth &amp; exit-multiple)</t>
+          <t>DCF value (avg of Gordon-growth, exit-multiple &amp; 3-stage to FY2040)</t>
         </is>
       </c>
       <c r="B77" s="41">
-        <f>AVERAGE(B38,B76)</f>
-        <v/>
+        <f>AVERAGE(B38,B76,B94)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="18" t="inlineStr">
+        <is>
+          <t>Extended forecast - Stage 2 fade (FY34-FY40): 3-stage DCF</t>
+        </is>
+      </c>
+      <c r="B80" s="19" t="n"/>
+      <c r="C80" s="19" t="n"/>
+      <c r="D80" s="19" t="n"/>
+      <c r="E80" s="19" t="n"/>
+      <c r="F80" s="19" t="n"/>
+      <c r="G80" s="19" t="n"/>
+      <c r="H80" s="19" t="n"/>
+    </row>
+    <row r="81">
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>FY2034E</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>FY2035E</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>FY2036E</t>
+        </is>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>FY2037E</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>FY2038E</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
+          <t>FY2039E</t>
+        </is>
+      </c>
+      <c r="H81" s="5" t="inlineStr">
+        <is>
+          <t>FY2040E</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="inlineStr">
+        <is>
+          <t>Fade growth in FCFF (%)</t>
+        </is>
+      </c>
+      <c r="B82" s="76" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C82" s="76" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="D82" s="76" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E82" s="76" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="F82" s="76" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="G82" s="76" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H82" s="76" t="n">
+        <v>0.055</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>Free cash flow to firm (FCFF)</t>
+        </is>
+      </c>
+      <c r="B83" s="77">
+        <f>H26*(1+B82)</f>
+        <v/>
+      </c>
+      <c r="C83" s="77">
+        <f>B83*(1+C82)</f>
+        <v/>
+      </c>
+      <c r="D83" s="77">
+        <f>C83*(1+D82)</f>
+        <v/>
+      </c>
+      <c r="E83" s="77">
+        <f>D83*(1+E82)</f>
+        <v/>
+      </c>
+      <c r="F83" s="77">
+        <f>E83*(1+F82)</f>
+        <v/>
+      </c>
+      <c r="G83" s="77">
+        <f>F83*(1+G82)</f>
+        <v/>
+      </c>
+      <c r="H83" s="77">
+        <f>G83*(1+H82)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="11" t="inlineStr">
+        <is>
+          <t>Discount period</t>
+        </is>
+      </c>
+      <c r="B84" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="C84" s="39" t="n">
+        <v>9</v>
+      </c>
+      <c r="D84" s="39" t="n">
+        <v>10</v>
+      </c>
+      <c r="E84" s="39" t="n">
+        <v>11</v>
+      </c>
+      <c r="F84" s="39" t="n">
+        <v>12</v>
+      </c>
+      <c r="G84" s="39" t="n">
+        <v>13</v>
+      </c>
+      <c r="H84" s="39" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="11" t="inlineStr">
+        <is>
+          <t>Discount factor</t>
+        </is>
+      </c>
+      <c r="B85" s="40">
+        <f>1/(1+$B$16)^B84</f>
+        <v/>
+      </c>
+      <c r="C85" s="40">
+        <f>1/(1+$B$16)^C84</f>
+        <v/>
+      </c>
+      <c r="D85" s="40">
+        <f>1/(1+$B$16)^D84</f>
+        <v/>
+      </c>
+      <c r="E85" s="40">
+        <f>1/(1+$B$16)^E84</f>
+        <v/>
+      </c>
+      <c r="F85" s="40">
+        <f>1/(1+$B$16)^F84</f>
+        <v/>
+      </c>
+      <c r="G85" s="40">
+        <f>1/(1+$B$16)^G84</f>
+        <v/>
+      </c>
+      <c r="H85" s="40">
+        <f>1/(1+$B$16)^H84</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
+          <t>PV of FCFF</t>
+        </is>
+      </c>
+      <c r="B86" s="77">
+        <f>B83*B85</f>
+        <v/>
+      </c>
+      <c r="C86" s="77">
+        <f>C83*C85</f>
+        <v/>
+      </c>
+      <c r="D86" s="77">
+        <f>D83*D85</f>
+        <v/>
+      </c>
+      <c r="E86" s="77">
+        <f>E83*E85</f>
+        <v/>
+      </c>
+      <c r="F86" s="77">
+        <f>F83*F85</f>
+        <v/>
+      </c>
+      <c r="G86" s="77">
+        <f>G83*G85</f>
+        <v/>
+      </c>
+      <c r="H86" s="77">
+        <f>H83*H85</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="11" t="inlineStr">
+        <is>
+          <t>PV of Stage-1 FCFF (FY27-FY33)</t>
+        </is>
+      </c>
+      <c r="B88" s="68">
+        <f>B31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="11" t="inlineStr">
+        <is>
+          <t>PV of Stage-2 FCFF (FY34-FY40)</t>
+        </is>
+      </c>
+      <c r="B89" s="68">
+        <f>SUM(B86:H86)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="11" t="inlineStr">
+        <is>
+          <t>Terminal value from FY40 = FCFF(FY40) x (1+g)/(WACC-g)</t>
+        </is>
+      </c>
+      <c r="B90" s="68">
+        <f>H83*(1+B17)/(B16-B17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="11" t="inlineStr">
+        <is>
+          <t>PV of terminal value</t>
+        </is>
+      </c>
+      <c r="B91" s="68">
+        <f>B90*H85</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="inlineStr">
+        <is>
+          <t>Enterprise value (3-stage, to FY2040)</t>
+        </is>
+      </c>
+      <c r="B92" s="92">
+        <f>B88+B89+B91</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="11" t="inlineStr">
+        <is>
+          <t>Equity value (3-stage)</t>
+        </is>
+      </c>
+      <c r="B93" s="68">
+        <f>B92-B35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="6" t="inlineStr">
+        <is>
+          <t>Intrinsic value/share - 3-stage to FY2040 (Rs)</t>
+        </is>
+      </c>
+      <c r="B94" s="41">
+        <f>B93/B37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="9" t="inlineStr">
+        <is>
+          <t>Terminal value as % of EV (3-stage)</t>
+        </is>
+      </c>
+      <c r="B95" s="10">
+        <f>B91/B92</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="47" t="inlineStr">
+        <is>
+          <t>Memo: 2-stage Gordon = B38; exit-multiple = B76; 3-stage(2040) = B94</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Extend integrated forecast to FY2036 (10-yr) + rework DCF horizon
- Full three-statement model now forecasts FY27-FY36 (10 years) across
  P&L, Balance Sheet, Cash Flow, schedules and ratios; balances under
  all scenarios.
- DCF: explicit FCFF FY27-36, Stage-2 fade FY37-40, terminal from FY40;
  Gordon value rises to ~Rs3,210 as more growth is captured explicitly.
- Relative valuation retains forward (FY27E) P/E, EV/EBITDA and EV/Sales
  on the peer median; charts and Summary extended to FY36.
</commit_message>
<xml_diff>
--- a/Navin Fluorine International - Financial Model.xlsx
+++ b/Navin Fluorine International - Financial Model.xlsx
@@ -548,7 +548,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Revenue &amp; EBITDA (Rs Cr), FY21-FY33</a:t>
+              <a:t>Revenue &amp; EBITDA (Rs Cr), FY21-FY36</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -573,12 +573,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Summary'!$B$19:$N$19</f>
+              <f>'Summary'!$B$19:$Q$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$B$20:$N$20</f>
+              <f>'Summary'!$B$20:$Q$20</f>
             </numRef>
           </val>
         </ser>
@@ -597,12 +597,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Summary'!$B$19:$N$19</f>
+              <f>'Summary'!$B$19:$Q$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$B$21:$N$21</f>
+              <f>'Summary'!$B$21:$Q$21</f>
             </numRef>
           </val>
         </ser>
@@ -654,7 +654,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>PAT (Rs Cr), FY21-FY33</a:t>
+              <a:t>PAT (Rs Cr), FY21-FY36</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -679,12 +679,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Summary'!$B$19:$N$19</f>
+              <f>'Summary'!$B$19:$Q$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$B$24:$N$24</f>
+              <f>'Summary'!$B$24:$Q$24</f>
             </numRef>
           </val>
         </ser>
@@ -807,7 +807,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>FCFF (Rs Cr), FY27-FY33</a:t>
+              <a:t>FCFF (Rs Cr), FY27-FY36</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -827,7 +827,7 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'DCF'!$B$19:$H$19</f>
+              <f>'DCF'!$B$19:$K$19</f>
             </numRef>
           </cat>
           <val>
@@ -846,7 +846,7 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'DCF'!$B$19:$H$19</f>
+              <f>'DCF'!$B$19:$K$19</f>
             </numRef>
           </cat>
           <val>
@@ -865,7 +865,7 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'DCF'!$B$19:$H$19</f>
+              <f>'DCF'!$B$19:$K$19</f>
             </numRef>
           </cat>
           <val>
@@ -884,7 +884,7 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'DCF'!$B$19:$H$19</f>
+              <f>'DCF'!$B$19:$K$19</f>
             </numRef>
           </cat>
           <val>
@@ -903,7 +903,7 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'DCF'!$B$19:$H$19</f>
+              <f>'DCF'!$B$19:$K$19</f>
             </numRef>
           </cat>
           <val>
@@ -922,7 +922,7 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'DCF'!$B$19:$H$19</f>
+              <f>'DCF'!$B$19:$K$19</f>
             </numRef>
           </cat>
           <val>
@@ -941,12 +941,69 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'DCF'!$B$19:$H$19</f>
+              <f>'DCF'!$B$19:$K$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
               <f>'DCF'!$H$26</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'DCF'!$B$19:$K$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'DCF'!$I$26</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="8"/>
+          <order val="8"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'DCF'!$B$19:$K$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'DCF'!$J$26</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="9"/>
+          <order val="9"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'DCF'!$B$19:$K$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'DCF'!$K$26</f>
             </numRef>
           </val>
         </ser>
@@ -1375,7 +1432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N38"/>
+  <dimension ref="A1:Q38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1392,6 +1449,9 @@
     <col width="12.5" customWidth="1" min="12" max="12"/>
     <col width="12.5" customWidth="1" min="13" max="13"/>
     <col width="12.5" customWidth="1" min="14" max="14"/>
+    <col width="12.5" customWidth="1" min="15" max="15"/>
+    <col width="12.5" customWidth="1" min="16" max="16"/>
+    <col width="12.5" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -1413,6 +1473,9 @@
       <c r="L1" s="2" t="n"/>
       <c r="M1" s="2" t="n"/>
       <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -1716,6 +1779,21 @@
           <t>FY2033E</t>
         </is>
       </c>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>FY2034E</t>
+        </is>
+      </c>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>FY2035E</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>FY2036E</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -1775,6 +1853,18 @@
         <f>'Profit &amp; Loss'!N4</f>
         <v/>
       </c>
+      <c r="O20" s="67">
+        <f>'Profit &amp; Loss'!O4</f>
+        <v/>
+      </c>
+      <c r="P20" s="67">
+        <f>'Profit &amp; Loss'!P4</f>
+        <v/>
+      </c>
+      <c r="Q20" s="67">
+        <f>'Profit &amp; Loss'!Q4</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -1834,6 +1924,18 @@
         <f>'Profit &amp; Loss'!N10</f>
         <v/>
       </c>
+      <c r="O21" s="67">
+        <f>'Profit &amp; Loss'!O10</f>
+        <v/>
+      </c>
+      <c r="P21" s="67">
+        <f>'Profit &amp; Loss'!P10</f>
+        <v/>
+      </c>
+      <c r="Q21" s="67">
+        <f>'Profit &amp; Loss'!Q10</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
@@ -1893,6 +1995,18 @@
         <f>'Profit &amp; Loss'!N11</f>
         <v/>
       </c>
+      <c r="O22" s="23">
+        <f>'Profit &amp; Loss'!O11</f>
+        <v/>
+      </c>
+      <c r="P22" s="23">
+        <f>'Profit &amp; Loss'!P11</f>
+        <v/>
+      </c>
+      <c r="Q22" s="23">
+        <f>'Profit &amp; Loss'!Q11</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
@@ -1952,6 +2066,18 @@
         <f>'Profit &amp; Loss'!N13</f>
         <v/>
       </c>
+      <c r="O23" s="30">
+        <f>'Profit &amp; Loss'!O13</f>
+        <v/>
+      </c>
+      <c r="P23" s="30">
+        <f>'Profit &amp; Loss'!P13</f>
+        <v/>
+      </c>
+      <c r="Q23" s="30">
+        <f>'Profit &amp; Loss'!Q13</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -2011,6 +2137,18 @@
         <f>'Profit &amp; Loss'!N21</f>
         <v/>
       </c>
+      <c r="O24" s="67">
+        <f>'Profit &amp; Loss'!O21</f>
+        <v/>
+      </c>
+      <c r="P24" s="67">
+        <f>'Profit &amp; Loss'!P21</f>
+        <v/>
+      </c>
+      <c r="Q24" s="67">
+        <f>'Profit &amp; Loss'!Q21</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
@@ -2070,6 +2208,18 @@
         <f>'Profit &amp; Loss'!N22</f>
         <v/>
       </c>
+      <c r="O25" s="16">
+        <f>'Profit &amp; Loss'!O22</f>
+        <v/>
+      </c>
+      <c r="P25" s="16">
+        <f>'Profit &amp; Loss'!P22</f>
+        <v/>
+      </c>
+      <c r="Q25" s="16">
+        <f>'Profit &amp; Loss'!Q22</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
@@ -2129,6 +2279,18 @@
         <f>'Ratio Analysis'!N17</f>
         <v/>
       </c>
+      <c r="O26" s="23">
+        <f>'Ratio Analysis'!O17</f>
+        <v/>
+      </c>
+      <c r="P26" s="23">
+        <f>'Ratio Analysis'!P17</f>
+        <v/>
+      </c>
+      <c r="Q26" s="23">
+        <f>'Ratio Analysis'!Q17</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
@@ -2188,6 +2350,18 @@
         <f>'Ratio Analysis'!N18</f>
         <v/>
       </c>
+      <c r="O27" s="23">
+        <f>'Ratio Analysis'!O18</f>
+        <v/>
+      </c>
+      <c r="P27" s="23">
+        <f>'Ratio Analysis'!P18</f>
+        <v/>
+      </c>
+      <c r="Q27" s="23">
+        <f>'Ratio Analysis'!Q18</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
@@ -2245,6 +2419,18 @@
       </c>
       <c r="N28" s="30">
         <f>'Working Schedules'!N28</f>
+        <v/>
+      </c>
+      <c r="O28" s="30">
+        <f>'Working Schedules'!O28</f>
+        <v/>
+      </c>
+      <c r="P28" s="30">
+        <f>'Working Schedules'!P28</f>
+        <v/>
+      </c>
+      <c r="Q28" s="30">
+        <f>'Working Schedules'!Q28</f>
         <v/>
       </c>
     </row>
@@ -2286,6 +2472,18 @@
       </c>
       <c r="N29" s="30">
         <f>DCF!H26</f>
+        <v/>
+      </c>
+      <c r="O29" s="30">
+        <f>DCF!I26</f>
+        <v/>
+      </c>
+      <c r="P29" s="30">
+        <f>DCF!J26</f>
+        <v/>
+      </c>
+      <c r="Q29" s="30">
+        <f>DCF!K26</f>
         <v/>
       </c>
     </row>
@@ -2372,7 +2570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N42"/>
+  <dimension ref="A1:Q42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2389,6 +2587,9 @@
     <col width="12.5" customWidth="1" min="12" max="12"/>
     <col width="12.5" customWidth="1" min="13" max="13"/>
     <col width="12.5" customWidth="1" min="14" max="14"/>
+    <col width="12.5" customWidth="1" min="15" max="15"/>
+    <col width="12.5" customWidth="1" min="16" max="16"/>
+    <col width="12.5" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -2410,6 +2611,9 @@
       <c r="L1" s="2" t="n"/>
       <c r="M1" s="2" t="n"/>
       <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -2483,6 +2687,21 @@
       <c r="N3" s="35" t="inlineStr">
         <is>
           <t>FY2033E</t>
+        </is>
+      </c>
+      <c r="O3" s="35" t="inlineStr">
+        <is>
+          <t>FY2034E</t>
+        </is>
+      </c>
+      <c r="P3" s="35" t="inlineStr">
+        <is>
+          <t>FY2035E</t>
+        </is>
+      </c>
+      <c r="Q3" s="35" t="inlineStr">
+        <is>
+          <t>FY2036E</t>
         </is>
       </c>
     </row>
@@ -2505,6 +2724,9 @@
       <c r="L4" s="19" t="n"/>
       <c r="M4" s="19" t="n"/>
       <c r="N4" s="19" t="n"/>
+      <c r="O4" s="19" t="n"/>
+      <c r="P4" s="19" t="n"/>
+      <c r="Q4" s="19" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -2560,6 +2782,18 @@
         <f>M8</f>
         <v/>
       </c>
+      <c r="O5" s="13">
+        <f>N8</f>
+        <v/>
+      </c>
+      <c r="P5" s="13">
+        <f>O8</f>
+        <v/>
+      </c>
+      <c r="Q5" s="13">
+        <f>P8</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
@@ -2619,6 +2853,18 @@
         <f>N5*Assumptions!N10</f>
         <v/>
       </c>
+      <c r="O6" s="13">
+        <f>O5*Assumptions!O10</f>
+        <v/>
+      </c>
+      <c r="P6" s="13">
+        <f>P5*Assumptions!P10</f>
+        <v/>
+      </c>
+      <c r="Q6" s="13">
+        <f>Q5*Assumptions!Q10</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
@@ -2674,6 +2920,18 @@
         <f>Assumptions!N11</f>
         <v/>
       </c>
+      <c r="O7" s="16">
+        <f>Assumptions!O11</f>
+        <v/>
+      </c>
+      <c r="P7" s="16">
+        <f>Assumptions!P11</f>
+        <v/>
+      </c>
+      <c r="Q7" s="16">
+        <f>Assumptions!Q11</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -2731,6 +2989,18 @@
       </c>
       <c r="N8" s="77">
         <f>N5-N6+N7</f>
+        <v/>
+      </c>
+      <c r="O8" s="77">
+        <f>O5-O6+O7</f>
+        <v/>
+      </c>
+      <c r="P8" s="77">
+        <f>P5-P6+P7</f>
+        <v/>
+      </c>
+      <c r="Q8" s="77">
+        <f>Q5-Q6+Q7</f>
         <v/>
       </c>
     </row>
@@ -2753,6 +3023,9 @@
       <c r="L10" s="19" t="n"/>
       <c r="M10" s="19" t="n"/>
       <c r="N10" s="19" t="n"/>
+      <c r="O10" s="19" t="n"/>
+      <c r="P10" s="19" t="n"/>
+      <c r="Q10" s="19" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
@@ -2808,6 +3081,18 @@
         <f>M12</f>
         <v/>
       </c>
+      <c r="O11" s="13">
+        <f>N12</f>
+        <v/>
+      </c>
+      <c r="P11" s="13">
+        <f>O12</f>
+        <v/>
+      </c>
+      <c r="Q11" s="13">
+        <f>P12</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -2867,6 +3152,18 @@
         <f>Assumptions!N19</f>
         <v/>
       </c>
+      <c r="O12" s="22">
+        <f>Assumptions!O19</f>
+        <v/>
+      </c>
+      <c r="P12" s="22">
+        <f>Assumptions!P19</f>
+        <v/>
+      </c>
+      <c r="Q12" s="22">
+        <f>Assumptions!Q19</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
@@ -2926,6 +3223,18 @@
         <f>(N11+N12)/2*Assumptions!N20</f>
         <v/>
       </c>
+      <c r="O13" s="13">
+        <f>(O11+O12)/2*Assumptions!O20</f>
+        <v/>
+      </c>
+      <c r="P13" s="13">
+        <f>(P11+P12)/2*Assumptions!P20</f>
+        <v/>
+      </c>
+      <c r="Q13" s="13">
+        <f>(Q11+Q12)/2*Assumptions!Q20</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -2983,6 +3292,18 @@
       </c>
       <c r="N14" s="10">
         <f>IF(N11=0,"",N13/((N11+N12)/2))</f>
+        <v/>
+      </c>
+      <c r="O14" s="10">
+        <f>IF(O11=0,"",O13/((O11+O12)/2))</f>
+        <v/>
+      </c>
+      <c r="P14" s="10">
+        <f>IF(P11=0,"",P13/((P11+P12)/2))</f>
+        <v/>
+      </c>
+      <c r="Q14" s="10">
+        <f>IF(Q11=0,"",Q13/((Q11+Q12)/2))</f>
         <v/>
       </c>
     </row>
@@ -3005,6 +3326,9 @@
       <c r="L16" s="19" t="n"/>
       <c r="M16" s="19" t="n"/>
       <c r="N16" s="19" t="n"/>
+      <c r="O16" s="19" t="n"/>
+      <c r="P16" s="19" t="n"/>
+      <c r="Q16" s="19" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
@@ -3060,6 +3384,18 @@
         <f>M21</f>
         <v/>
       </c>
+      <c r="O17" s="13">
+        <f>N21</f>
+        <v/>
+      </c>
+      <c r="P17" s="13">
+        <f>O21</f>
+        <v/>
+      </c>
+      <c r="Q17" s="13">
+        <f>P21</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
@@ -3119,6 +3455,18 @@
         <f>'Profit &amp; Loss'!N21</f>
         <v/>
       </c>
+      <c r="O18" s="16">
+        <f>'Profit &amp; Loss'!O21</f>
+        <v/>
+      </c>
+      <c r="P18" s="16">
+        <f>'Profit &amp; Loss'!P21</f>
+        <v/>
+      </c>
+      <c r="Q18" s="16">
+        <f>'Profit &amp; Loss'!Q21</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
@@ -3174,6 +3522,18 @@
         <f>N41</f>
         <v/>
       </c>
+      <c r="O19" s="16">
+        <f>O41</f>
+        <v/>
+      </c>
+      <c r="P19" s="16">
+        <f>P41</f>
+        <v/>
+      </c>
+      <c r="Q19" s="16">
+        <f>Q41</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
@@ -3218,6 +3578,15 @@
       <c r="N20" s="12" t="n">
         <v>0</v>
       </c>
+      <c r="O20" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -3277,6 +3646,18 @@
         <f>N17+N18-N19+N20</f>
         <v/>
       </c>
+      <c r="O21" s="77">
+        <f>O17+O18-O19+O20</f>
+        <v/>
+      </c>
+      <c r="P21" s="77">
+        <f>P17+P18-P19+P20</f>
+        <v/>
+      </c>
+      <c r="Q21" s="77">
+        <f>Q17+Q18-Q19+Q20</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
@@ -3336,6 +3717,18 @@
         <f>M22</f>
         <v/>
       </c>
+      <c r="O22" s="13">
+        <f>N22</f>
+        <v/>
+      </c>
+      <c r="P22" s="13">
+        <f>O22</f>
+        <v/>
+      </c>
+      <c r="Q22" s="13">
+        <f>P22</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
@@ -3393,6 +3786,18 @@
       </c>
       <c r="N23" s="13">
         <f>N22/2</f>
+        <v/>
+      </c>
+      <c r="O23" s="13">
+        <f>O22/2</f>
+        <v/>
+      </c>
+      <c r="P23" s="13">
+        <f>P22/2</f>
+        <v/>
+      </c>
+      <c r="Q23" s="13">
+        <f>Q22/2</f>
         <v/>
       </c>
     </row>
@@ -3415,6 +3820,9 @@
       <c r="L25" s="19" t="n"/>
       <c r="M25" s="19" t="n"/>
       <c r="N25" s="19" t="n"/>
+      <c r="O25" s="19" t="n"/>
+      <c r="P25" s="19" t="n"/>
+      <c r="Q25" s="19" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
@@ -3474,6 +3882,18 @@
         <f>'Balance Sheet'!N18</f>
         <v/>
       </c>
+      <c r="O26" s="16">
+        <f>'Balance Sheet'!O18</f>
+        <v/>
+      </c>
+      <c r="P26" s="16">
+        <f>'Balance Sheet'!P18</f>
+        <v/>
+      </c>
+      <c r="Q26" s="16">
+        <f>'Balance Sheet'!Q18</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
@@ -3533,6 +3953,18 @@
         <f>'Balance Sheet'!N11</f>
         <v/>
       </c>
+      <c r="O27" s="16">
+        <f>'Balance Sheet'!O11</f>
+        <v/>
+      </c>
+      <c r="P27" s="16">
+        <f>'Balance Sheet'!P11</f>
+        <v/>
+      </c>
+      <c r="Q27" s="16">
+        <f>'Balance Sheet'!Q11</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -3590,6 +4022,18 @@
       </c>
       <c r="N28" s="77">
         <f>N26-N27</f>
+        <v/>
+      </c>
+      <c r="O28" s="77">
+        <f>O26-O27</f>
+        <v/>
+      </c>
+      <c r="P28" s="77">
+        <f>P26-P27</f>
+        <v/>
+      </c>
+      <c r="Q28" s="77">
+        <f>Q26-Q27</f>
         <v/>
       </c>
     </row>
@@ -3640,6 +4084,15 @@
       <c r="N31" s="51" t="n">
         <v>0.15</v>
       </c>
+      <c r="O31" s="51" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P31" s="51" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q31" s="51" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
@@ -3675,6 +4128,18 @@
         <f>N31*'Profit &amp; Loss'!N4</f>
         <v/>
       </c>
+      <c r="O32" s="13">
+        <f>O31*'Profit &amp; Loss'!O4</f>
+        <v/>
+      </c>
+      <c r="P32" s="13">
+        <f>P31*'Profit &amp; Loss'!P4</f>
+        <v/>
+      </c>
+      <c r="Q32" s="13">
+        <f>Q31*'Profit &amp; Loss'!Q4</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
@@ -3710,6 +4175,18 @@
         <f>'Balance Sheet'!M11</f>
         <v/>
       </c>
+      <c r="O33" s="16">
+        <f>'Balance Sheet'!N11</f>
+        <v/>
+      </c>
+      <c r="P33" s="16">
+        <f>'Balance Sheet'!O11</f>
+        <v/>
+      </c>
+      <c r="Q33" s="16">
+        <f>'Balance Sheet'!P11</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
@@ -3745,6 +4222,18 @@
         <f>'Profit &amp; Loss'!N21</f>
         <v/>
       </c>
+      <c r="O34" s="16">
+        <f>'Profit &amp; Loss'!O21</f>
+        <v/>
+      </c>
+      <c r="P34" s="16">
+        <f>'Profit &amp; Loss'!P21</f>
+        <v/>
+      </c>
+      <c r="Q34" s="16">
+        <f>'Profit &amp; Loss'!Q21</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
@@ -3780,6 +4269,18 @@
         <f>'Profit &amp; Loss'!N12</f>
         <v/>
       </c>
+      <c r="O35" s="16">
+        <f>'Profit &amp; Loss'!O12</f>
+        <v/>
+      </c>
+      <c r="P35" s="16">
+        <f>'Profit &amp; Loss'!P12</f>
+        <v/>
+      </c>
+      <c r="Q35" s="16">
+        <f>'Profit &amp; Loss'!Q12</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
@@ -3815,6 +4316,18 @@
         <f>'Working Capital Schedule'!N12</f>
         <v/>
       </c>
+      <c r="O36" s="16">
+        <f>'Working Capital Schedule'!O12</f>
+        <v/>
+      </c>
+      <c r="P36" s="16">
+        <f>'Working Capital Schedule'!P12</f>
+        <v/>
+      </c>
+      <c r="Q36" s="16">
+        <f>'Working Capital Schedule'!Q12</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
@@ -3850,6 +4363,18 @@
         <f>Assumptions!N11</f>
         <v/>
       </c>
+      <c r="O37" s="16">
+        <f>Assumptions!O11</f>
+        <v/>
+      </c>
+      <c r="P37" s="16">
+        <f>Assumptions!P11</f>
+        <v/>
+      </c>
+      <c r="Q37" s="16">
+        <f>Assumptions!Q11</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
@@ -3885,6 +4410,18 @@
         <f>N12-N11</f>
         <v/>
       </c>
+      <c r="O38" s="13">
+        <f>O12-O11</f>
+        <v/>
+      </c>
+      <c r="P38" s="13">
+        <f>P12-P11</f>
+        <v/>
+      </c>
+      <c r="Q38" s="13">
+        <f>Q12-Q11</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
@@ -3920,6 +4457,18 @@
         <f>N33+N34+N35-N36-N37+N38+N20</f>
         <v/>
       </c>
+      <c r="O39" s="77">
+        <f>O33+O34+O35-O36-O37+O38+O20</f>
+        <v/>
+      </c>
+      <c r="P39" s="77">
+        <f>P33+P34+P35-P36-P37+P38+P20</f>
+        <v/>
+      </c>
+      <c r="Q39" s="77">
+        <f>Q33+Q34+Q35-Q36-Q37+Q38+Q20</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="11" t="inlineStr">
@@ -3955,6 +4504,18 @@
         <f>'Profit &amp; Loss'!N21*Assumptions!N13</f>
         <v/>
       </c>
+      <c r="O40" s="13">
+        <f>'Profit &amp; Loss'!O21*Assumptions!O13</f>
+        <v/>
+      </c>
+      <c r="P40" s="13">
+        <f>'Profit &amp; Loss'!P21*Assumptions!P13</f>
+        <v/>
+      </c>
+      <c r="Q40" s="13">
+        <f>'Profit &amp; Loss'!Q21*Assumptions!Q13</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
@@ -3990,6 +4551,18 @@
         <f>MAX(N40,N39-N32)</f>
         <v/>
       </c>
+      <c r="O41" s="77">
+        <f>MAX(O40,O39-O32)</f>
+        <v/>
+      </c>
+      <c r="P41" s="77">
+        <f>MAX(P40,P39-P32)</f>
+        <v/>
+      </c>
+      <c r="Q41" s="77">
+        <f>MAX(Q40,Q39-Q32)</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
@@ -4023,6 +4596,18 @@
       </c>
       <c r="N42" s="15">
         <f>N39-N41</f>
+        <v/>
+      </c>
+      <c r="O42" s="15">
+        <f>O39-O41</f>
+        <v/>
+      </c>
+      <c r="P42" s="15">
+        <f>P39-P41</f>
+        <v/>
+      </c>
+      <c r="Q42" s="15">
+        <f>Q39-Q41</f>
         <v/>
       </c>
     </row>
@@ -4037,7 +4622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:Q26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4054,6 +4639,9 @@
     <col width="12.5" customWidth="1" min="12" max="12"/>
     <col width="12.5" customWidth="1" min="13" max="13"/>
     <col width="12.5" customWidth="1" min="14" max="14"/>
+    <col width="12.5" customWidth="1" min="15" max="15"/>
+    <col width="12.5" customWidth="1" min="16" max="16"/>
+    <col width="12.5" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -4075,6 +4663,9 @@
       <c r="L1" s="2" t="n"/>
       <c r="M1" s="2" t="n"/>
       <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -4356,7 +4947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N48"/>
+  <dimension ref="A1:Q48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4373,6 +4964,9 @@
     <col width="12.5" customWidth="1" min="12" max="12"/>
     <col width="12.5" customWidth="1" min="13" max="13"/>
     <col width="12.5" customWidth="1" min="14" max="14"/>
+    <col width="12.5" customWidth="1" min="15" max="15"/>
+    <col width="12.5" customWidth="1" min="16" max="16"/>
+    <col width="12.5" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -4394,6 +4988,9 @@
       <c r="L1" s="2" t="n"/>
       <c r="M1" s="2" t="n"/>
       <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -4471,6 +5068,21 @@
       <c r="N3" s="5" t="inlineStr">
         <is>
           <t>FY2033E</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>FY2034E</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>FY2035E</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>FY2036E</t>
         </is>
       </c>
     </row>
@@ -5131,6 +5743,9 @@
       <c r="L32" s="19" t="n"/>
       <c r="M32" s="19" t="n"/>
       <c r="N32" s="19" t="n"/>
+      <c r="O32" s="19" t="n"/>
+      <c r="P32" s="19" t="n"/>
+      <c r="Q32" s="19" t="n"/>
     </row>
     <row r="33" ht="58" customHeight="1">
       <c r="A33" s="31" t="inlineStr">
@@ -5283,7 +5898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N95"/>
+  <dimension ref="A1:Q95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5300,6 +5915,9 @@
     <col width="12.5" customWidth="1" min="12" max="12"/>
     <col width="12.5" customWidth="1" min="13" max="13"/>
     <col width="12.5" customWidth="1" min="14" max="14"/>
+    <col width="12.5" customWidth="1" min="15" max="15"/>
+    <col width="12.5" customWidth="1" min="16" max="16"/>
+    <col width="12.5" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -5321,6 +5939,9 @@
       <c r="L1" s="2" t="n"/>
       <c r="M1" s="2" t="n"/>
       <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -6349,7 +6970,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N96"/>
+  <dimension ref="A1:Q96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -6366,6 +6987,9 @@
     <col width="12.5" customWidth="1" min="12" max="12"/>
     <col width="12.5" customWidth="1" min="13" max="13"/>
     <col width="12.5" customWidth="1" min="14" max="14"/>
+    <col width="12.5" customWidth="1" min="15" max="15"/>
+    <col width="12.5" customWidth="1" min="16" max="16"/>
+    <col width="12.5" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -6387,6 +7011,9 @@
       <c r="L1" s="2" t="n"/>
       <c r="M1" s="2" t="n"/>
       <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -6594,6 +7221,21 @@
           <t>FY2033E</t>
         </is>
       </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>FY2034E</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>FY2035E</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>FY2036E</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
@@ -6629,6 +7271,18 @@
         <f>'Profit &amp; Loss'!N13</f>
         <v/>
       </c>
+      <c r="I20" s="16">
+        <f>'Profit &amp; Loss'!O13</f>
+        <v/>
+      </c>
+      <c r="J20" s="16">
+        <f>'Profit &amp; Loss'!P13</f>
+        <v/>
+      </c>
+      <c r="K20" s="16">
+        <f>'Profit &amp; Loss'!Q13</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
@@ -6664,6 +7318,18 @@
         <f>H20*$B$10</f>
         <v/>
       </c>
+      <c r="I21" s="13">
+        <f>I20*$B$10</f>
+        <v/>
+      </c>
+      <c r="J21" s="13">
+        <f>J20*$B$10</f>
+        <v/>
+      </c>
+      <c r="K21" s="13">
+        <f>K20*$B$10</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
@@ -6699,6 +7365,18 @@
         <f>H20-H21</f>
         <v/>
       </c>
+      <c r="I22" s="77">
+        <f>I20-I21</f>
+        <v/>
+      </c>
+      <c r="J22" s="77">
+        <f>J20-J21</f>
+        <v/>
+      </c>
+      <c r="K22" s="77">
+        <f>K20-K21</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
@@ -6734,6 +7412,18 @@
         <f>'Profit &amp; Loss'!N12</f>
         <v/>
       </c>
+      <c r="I23" s="16">
+        <f>'Profit &amp; Loss'!O12</f>
+        <v/>
+      </c>
+      <c r="J23" s="16">
+        <f>'Profit &amp; Loss'!P12</f>
+        <v/>
+      </c>
+      <c r="K23" s="16">
+        <f>'Profit &amp; Loss'!Q12</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
@@ -6769,6 +7459,18 @@
         <f>Assumptions!N11</f>
         <v/>
       </c>
+      <c r="I24" s="16">
+        <f>Assumptions!O11</f>
+        <v/>
+      </c>
+      <c r="J24" s="16">
+        <f>Assumptions!P11</f>
+        <v/>
+      </c>
+      <c r="K24" s="16">
+        <f>Assumptions!Q11</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
@@ -6804,6 +7506,18 @@
         <f>'Working Capital Schedule'!N12</f>
         <v/>
       </c>
+      <c r="I25" s="16">
+        <f>'Working Capital Schedule'!O12</f>
+        <v/>
+      </c>
+      <c r="J25" s="16">
+        <f>'Working Capital Schedule'!P12</f>
+        <v/>
+      </c>
+      <c r="K25" s="16">
+        <f>'Working Capital Schedule'!Q12</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
@@ -6839,6 +7553,18 @@
         <f>H22+H23-H24-H25</f>
         <v/>
       </c>
+      <c r="I26" s="15">
+        <f>I22+I23-I24-I25</f>
+        <v/>
+      </c>
+      <c r="J26" s="15">
+        <f>J22+J23-J24-J25</f>
+        <v/>
+      </c>
+      <c r="K26" s="15">
+        <f>K22+K23-K24-K25</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
@@ -6867,6 +7593,15 @@
       <c r="H27" s="39" t="n">
         <v>7</v>
       </c>
+      <c r="I27" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="J27" s="39" t="n">
+        <v>9</v>
+      </c>
+      <c r="K27" s="39" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
@@ -6902,6 +7637,18 @@
         <f>1/(1+$B$16)^H27</f>
         <v/>
       </c>
+      <c r="I28" s="40">
+        <f>1/(1+$B$16)^I27</f>
+        <v/>
+      </c>
+      <c r="J28" s="40">
+        <f>1/(1+$B$16)^J27</f>
+        <v/>
+      </c>
+      <c r="K28" s="40">
+        <f>1/(1+$B$16)^K27</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
@@ -6937,6 +7684,18 @@
         <f>H26*H28</f>
         <v/>
       </c>
+      <c r="I29" s="77">
+        <f>I26*I28</f>
+        <v/>
+      </c>
+      <c r="J29" s="77">
+        <f>J26*J28</f>
+        <v/>
+      </c>
+      <c r="K29" s="77">
+        <f>K26*K28</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
@@ -6945,7 +7704,7 @@
         </is>
       </c>
       <c r="B31" s="77">
-        <f>SUM(B29:H29)</f>
+        <f>SUM(B29:K29)</f>
         <v/>
       </c>
     </row>
@@ -6956,7 +7715,7 @@
         </is>
       </c>
       <c r="B32" s="13">
-        <f>H26*(1+B17)/(B16-B17)</f>
+        <f>K26*(1+B17)/(B16-B17)</f>
         <v/>
       </c>
     </row>
@@ -6967,7 +7726,7 @@
         </is>
       </c>
       <c r="B33" s="13">
-        <f>B32*H28</f>
+        <f>B32*K28</f>
         <v/>
       </c>
     </row>
@@ -7098,23 +7857,23 @@
         <v>0.11</v>
       </c>
       <c r="B46" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A46)^(-$B$27:$H$27))+($H$26*(1+B$45)/($A46-B$45))*(1+$A46)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A46)^(-$B$27:$K$27))+($K$26*(1+B$45)/($A46-B$45))*(1+$A46)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="C46" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A46)^(-$B$27:$H$27))+($H$26*(1+C$45)/($A46-C$45))*(1+$A46)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A46)^(-$B$27:$K$27))+($K$26*(1+C$45)/($A46-C$45))*(1+$A46)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="D46" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A46)^(-$B$27:$H$27))+($H$26*(1+D$45)/($A46-D$45))*(1+$A46)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A46)^(-$B$27:$K$27))+($K$26*(1+D$45)/($A46-D$45))*(1+$A46)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="E46" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A46)^(-$B$27:$H$27))+($H$26*(1+E$45)/($A46-E$45))*(1+$A46)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A46)^(-$B$27:$K$27))+($K$26*(1+E$45)/($A46-E$45))*(1+$A46)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="F46" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A46)^(-$B$27:$H$27))+($H$26*(1+F$45)/($A46-F$45))*(1+$A46)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A46)^(-$B$27:$K$27))+($K$26*(1+F$45)/($A46-F$45))*(1+$A46)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
     </row>
@@ -7123,23 +7882,23 @@
         <v>0.115</v>
       </c>
       <c r="B47" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A47)^(-$B$27:$H$27))+($H$26*(1+B$45)/($A47-B$45))*(1+$A47)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A47)^(-$B$27:$K$27))+($K$26*(1+B$45)/($A47-B$45))*(1+$A47)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="C47" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A47)^(-$B$27:$H$27))+($H$26*(1+C$45)/($A47-C$45))*(1+$A47)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A47)^(-$B$27:$K$27))+($K$26*(1+C$45)/($A47-C$45))*(1+$A47)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="D47" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A47)^(-$B$27:$H$27))+($H$26*(1+D$45)/($A47-D$45))*(1+$A47)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A47)^(-$B$27:$K$27))+($K$26*(1+D$45)/($A47-D$45))*(1+$A47)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="E47" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A47)^(-$B$27:$H$27))+($H$26*(1+E$45)/($A47-E$45))*(1+$A47)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A47)^(-$B$27:$K$27))+($K$26*(1+E$45)/($A47-E$45))*(1+$A47)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="F47" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A47)^(-$B$27:$H$27))+($H$26*(1+F$45)/($A47-F$45))*(1+$A47)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A47)^(-$B$27:$K$27))+($K$26*(1+F$45)/($A47-F$45))*(1+$A47)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
     </row>
@@ -7148,23 +7907,23 @@
         <v>0.12</v>
       </c>
       <c r="B48" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A48)^(-$B$27:$H$27))+($H$26*(1+B$45)/($A48-B$45))*(1+$A48)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A48)^(-$B$27:$K$27))+($K$26*(1+B$45)/($A48-B$45))*(1+$A48)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="C48" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A48)^(-$B$27:$H$27))+($H$26*(1+C$45)/($A48-C$45))*(1+$A48)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A48)^(-$B$27:$K$27))+($K$26*(1+C$45)/($A48-C$45))*(1+$A48)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="D48" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A48)^(-$B$27:$H$27))+($H$26*(1+D$45)/($A48-D$45))*(1+$A48)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A48)^(-$B$27:$K$27))+($K$26*(1+D$45)/($A48-D$45))*(1+$A48)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="E48" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A48)^(-$B$27:$H$27))+($H$26*(1+E$45)/($A48-E$45))*(1+$A48)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A48)^(-$B$27:$K$27))+($K$26*(1+E$45)/($A48-E$45))*(1+$A48)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="F48" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A48)^(-$B$27:$H$27))+($H$26*(1+F$45)/($A48-F$45))*(1+$A48)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A48)^(-$B$27:$K$27))+($K$26*(1+F$45)/($A48-F$45))*(1+$A48)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
     </row>
@@ -7173,23 +7932,23 @@
         <v>0.125</v>
       </c>
       <c r="B49" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A49)^(-$B$27:$H$27))+($H$26*(1+B$45)/($A49-B$45))*(1+$A49)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A49)^(-$B$27:$K$27))+($K$26*(1+B$45)/($A49-B$45))*(1+$A49)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="C49" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A49)^(-$B$27:$H$27))+($H$26*(1+C$45)/($A49-C$45))*(1+$A49)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A49)^(-$B$27:$K$27))+($K$26*(1+C$45)/($A49-C$45))*(1+$A49)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="D49" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A49)^(-$B$27:$H$27))+($H$26*(1+D$45)/($A49-D$45))*(1+$A49)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A49)^(-$B$27:$K$27))+($K$26*(1+D$45)/($A49-D$45))*(1+$A49)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="E49" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A49)^(-$B$27:$H$27))+($H$26*(1+E$45)/($A49-E$45))*(1+$A49)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A49)^(-$B$27:$K$27))+($K$26*(1+E$45)/($A49-E$45))*(1+$A49)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="F49" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A49)^(-$B$27:$H$27))+($H$26*(1+F$45)/($A49-F$45))*(1+$A49)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A49)^(-$B$27:$K$27))+($K$26*(1+F$45)/($A49-F$45))*(1+$A49)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
     </row>
@@ -7198,23 +7957,23 @@
         <v>0.13</v>
       </c>
       <c r="B50" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A50)^(-$B$27:$H$27))+($H$26*(1+B$45)/($A50-B$45))*(1+$A50)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A50)^(-$B$27:$K$27))+($K$26*(1+B$45)/($A50-B$45))*(1+$A50)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="C50" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A50)^(-$B$27:$H$27))+($H$26*(1+C$45)/($A50-C$45))*(1+$A50)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A50)^(-$B$27:$K$27))+($K$26*(1+C$45)/($A50-C$45))*(1+$A50)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="D50" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A50)^(-$B$27:$H$27))+($H$26*(1+D$45)/($A50-D$45))*(1+$A50)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A50)^(-$B$27:$K$27))+($K$26*(1+D$45)/($A50-D$45))*(1+$A50)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="E50" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A50)^(-$B$27:$H$27))+($H$26*(1+E$45)/($A50-E$45))*(1+$A50)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A50)^(-$B$27:$K$27))+($K$26*(1+E$45)/($A50-E$45))*(1+$A50)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
       <c r="F50" s="44">
-        <f>(SUMPRODUCT($B$26:$H$26,(1+$A50)^(-$B$27:$H$27))+($H$26*(1+F$45)/($A50-F$45))*(1+$A50)^(-$H$27)-$B$35)/$B$37</f>
+        <f>(SUMPRODUCT($B$26:$K$26,(1+$A50)^(-$B$27:$K$27))+($K$26*(1+F$45)/($A50-F$45))*(1+$A50)^(-$K$27)-$B$35)/$B$37</f>
         <v/>
       </c>
     </row>
@@ -7241,11 +8000,11 @@
     <row r="71">
       <c r="A71" s="11" t="inlineStr">
         <is>
-          <t>Terminal-year (FY33) EBITDA</t>
+          <t>Terminal-year (FY36) EBITDA</t>
         </is>
       </c>
       <c r="B71" s="30">
-        <f>'Profit &amp; Loss'!N10</f>
+        <f>'Profit &amp; Loss'!Q10</f>
         <v/>
       </c>
     </row>
@@ -7267,7 +8026,7 @@
         </is>
       </c>
       <c r="B73" s="68">
-        <f>B72*H28</f>
+        <f>B72*K28</f>
         <v/>
       </c>
     </row>
@@ -7318,7 +8077,7 @@
     <row r="80">
       <c r="A80" s="18" t="inlineStr">
         <is>
-          <t>Extended forecast - Stage 2 fade (FY34-FY40): 3-stage DCF</t>
+          <t>Extended forecast - Stage 2 fade (FY37-FY40): 3-stage DCF</t>
         </is>
       </c>
       <c r="B80" s="19" t="n"/>
@@ -7332,35 +8091,20 @@
     <row r="81">
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>FY2034E</t>
+          <t>FY2037E</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>FY2035E</t>
+          <t>FY2038E</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>FY2036E</t>
+          <t>FY2039E</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
-        <is>
-          <t>FY2037E</t>
-        </is>
-      </c>
-      <c r="F81" s="5" t="inlineStr">
-        <is>
-          <t>FY2038E</t>
-        </is>
-      </c>
-      <c r="G81" s="5" t="inlineStr">
-        <is>
-          <t>FY2039E</t>
-        </is>
-      </c>
-      <c r="H81" s="5" t="inlineStr">
         <is>
           <t>FY2040E</t>
         </is>
@@ -7373,24 +8117,15 @@
         </is>
       </c>
       <c r="B82" s="76" t="n">
-        <v>0.1</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="C82" s="76" t="n">
-        <v>0.09</v>
+        <v>0.065</v>
       </c>
       <c r="D82" s="76" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="E82" s="76" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F82" s="76" t="n">
-        <v>0.065</v>
-      </c>
-      <c r="G82" s="76" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="H82" s="76" t="n">
         <v>0.055</v>
       </c>
     </row>
@@ -7401,7 +8136,7 @@
         </is>
       </c>
       <c r="B83" s="77">
-        <f>H26*(1+B82)</f>
+        <f>K26*(1+B82)</f>
         <v/>
       </c>
       <c r="C83" s="77">
@@ -7416,18 +8151,6 @@
         <f>D83*(1+E82)</f>
         <v/>
       </c>
-      <c r="F83" s="77">
-        <f>E83*(1+F82)</f>
-        <v/>
-      </c>
-      <c r="G83" s="77">
-        <f>F83*(1+G82)</f>
-        <v/>
-      </c>
-      <c r="H83" s="77">
-        <f>G83*(1+H82)</f>
-        <v/>
-      </c>
     </row>
     <row r="84">
       <c r="A84" s="11" t="inlineStr">
@@ -7436,24 +8159,15 @@
         </is>
       </c>
       <c r="B84" s="39" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C84" s="39" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D84" s="39" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E84" s="39" t="n">
-        <v>11</v>
-      </c>
-      <c r="F84" s="39" t="n">
-        <v>12</v>
-      </c>
-      <c r="G84" s="39" t="n">
-        <v>13</v>
-      </c>
-      <c r="H84" s="39" t="n">
         <v>14</v>
       </c>
     </row>
@@ -7479,18 +8193,6 @@
         <f>1/(1+$B$16)^E84</f>
         <v/>
       </c>
-      <c r="F85" s="40">
-        <f>1/(1+$B$16)^F84</f>
-        <v/>
-      </c>
-      <c r="G85" s="40">
-        <f>1/(1+$B$16)^G84</f>
-        <v/>
-      </c>
-      <c r="H85" s="40">
-        <f>1/(1+$B$16)^H84</f>
-        <v/>
-      </c>
     </row>
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
@@ -7514,18 +8216,6 @@
         <f>E83*E85</f>
         <v/>
       </c>
-      <c r="F86" s="77">
-        <f>F83*F85</f>
-        <v/>
-      </c>
-      <c r="G86" s="77">
-        <f>G83*G85</f>
-        <v/>
-      </c>
-      <c r="H86" s="77">
-        <f>H83*H85</f>
-        <v/>
-      </c>
     </row>
     <row r="88">
       <c r="A88" s="11" t="inlineStr">
@@ -7541,11 +8231,11 @@
     <row r="89">
       <c r="A89" s="11" t="inlineStr">
         <is>
-          <t>PV of Stage-2 FCFF (FY34-FY40)</t>
+          <t>PV of Stage-2 FCFF (FY37-FY40)</t>
         </is>
       </c>
       <c r="B89" s="68">
-        <f>SUM(B86:H86)</f>
+        <f>SUM(B86:E86)</f>
         <v/>
       </c>
     </row>
@@ -7556,7 +8246,7 @@
         </is>
       </c>
       <c r="B90" s="68">
-        <f>H83*(1+B17)/(B16-B17)</f>
+        <f>E83*(1+B17)/(B16-B17)</f>
         <v/>
       </c>
     </row>
@@ -7567,7 +8257,7 @@
         </is>
       </c>
       <c r="B91" s="68">
-        <f>B90*H85</f>
+        <f>B90*E85</f>
         <v/>
       </c>
     </row>
@@ -7634,7 +8324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -7651,6 +8341,9 @@
     <col width="12.5" customWidth="1" min="12" max="12"/>
     <col width="12.5" customWidth="1" min="13" max="13"/>
     <col width="12.5" customWidth="1" min="14" max="14"/>
+    <col width="12.5" customWidth="1" min="15" max="15"/>
+    <col width="12.5" customWidth="1" min="16" max="16"/>
+    <col width="12.5" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -7672,6 +8365,9 @@
       <c r="L1" s="2" t="n"/>
       <c r="M1" s="2" t="n"/>
       <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -7749,6 +8445,21 @@
       <c r="N3" s="5" t="inlineStr">
         <is>
           <t>FY2033E</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>FY2034E</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>FY2035E</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>FY2036E</t>
         </is>
       </c>
     </row>
@@ -7771,6 +8482,9 @@
       <c r="L4" s="19" t="n"/>
       <c r="M4" s="19" t="n"/>
       <c r="N4" s="19" t="n"/>
+      <c r="O4" s="19" t="n"/>
+      <c r="P4" s="19" t="n"/>
+      <c r="Q4" s="19" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -7826,6 +8540,18 @@
         <f>IF('Profit &amp; Loss'!M4=0,"",'Profit &amp; Loss'!N4/'Profit &amp; Loss'!M4-1)</f>
         <v/>
       </c>
+      <c r="O5" s="23">
+        <f>IF('Profit &amp; Loss'!N4=0,"",'Profit &amp; Loss'!O4/'Profit &amp; Loss'!N4-1)</f>
+        <v/>
+      </c>
+      <c r="P5" s="23">
+        <f>IF('Profit &amp; Loss'!O4=0,"",'Profit &amp; Loss'!P4/'Profit &amp; Loss'!O4-1)</f>
+        <v/>
+      </c>
+      <c r="Q5" s="23">
+        <f>IF('Profit &amp; Loss'!P4=0,"",'Profit &amp; Loss'!Q4/'Profit &amp; Loss'!P4-1)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
@@ -7881,6 +8607,18 @@
         <f>IF('Profit &amp; Loss'!M10=0,"",'Profit &amp; Loss'!N10/'Profit &amp; Loss'!M10-1)</f>
         <v/>
       </c>
+      <c r="O6" s="23">
+        <f>IF('Profit &amp; Loss'!N10=0,"",'Profit &amp; Loss'!O10/'Profit &amp; Loss'!N10-1)</f>
+        <v/>
+      </c>
+      <c r="P6" s="23">
+        <f>IF('Profit &amp; Loss'!O10=0,"",'Profit &amp; Loss'!P10/'Profit &amp; Loss'!O10-1)</f>
+        <v/>
+      </c>
+      <c r="Q6" s="23">
+        <f>IF('Profit &amp; Loss'!P10=0,"",'Profit &amp; Loss'!Q10/'Profit &amp; Loss'!P10-1)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
@@ -7936,6 +8674,18 @@
         <f>IF('Profit &amp; Loss'!M13=0,"",'Profit &amp; Loss'!N13/'Profit &amp; Loss'!M13-1)</f>
         <v/>
       </c>
+      <c r="O7" s="23">
+        <f>IF('Profit &amp; Loss'!N13=0,"",'Profit &amp; Loss'!O13/'Profit &amp; Loss'!N13-1)</f>
+        <v/>
+      </c>
+      <c r="P7" s="23">
+        <f>IF('Profit &amp; Loss'!O13=0,"",'Profit &amp; Loss'!P13/'Profit &amp; Loss'!O13-1)</f>
+        <v/>
+      </c>
+      <c r="Q7" s="23">
+        <f>IF('Profit &amp; Loss'!P13=0,"",'Profit &amp; Loss'!Q13/'Profit &amp; Loss'!P13-1)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
@@ -7989,6 +8739,18 @@
       </c>
       <c r="N8" s="23">
         <f>IF('Profit &amp; Loss'!M21=0,"",'Profit &amp; Loss'!N21/'Profit &amp; Loss'!M21-1)</f>
+        <v/>
+      </c>
+      <c r="O8" s="23">
+        <f>IF('Profit &amp; Loss'!N21=0,"",'Profit &amp; Loss'!O21/'Profit &amp; Loss'!N21-1)</f>
+        <v/>
+      </c>
+      <c r="P8" s="23">
+        <f>IF('Profit &amp; Loss'!O21=0,"",'Profit &amp; Loss'!P21/'Profit &amp; Loss'!O21-1)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="23">
+        <f>IF('Profit &amp; Loss'!P21=0,"",'Profit &amp; Loss'!Q21/'Profit &amp; Loss'!P21-1)</f>
         <v/>
       </c>
     </row>
@@ -8011,6 +8773,9 @@
       <c r="L10" s="19" t="n"/>
       <c r="M10" s="19" t="n"/>
       <c r="N10" s="19" t="n"/>
+      <c r="O10" s="19" t="n"/>
+      <c r="P10" s="19" t="n"/>
+      <c r="Q10" s="19" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
@@ -8070,6 +8835,18 @@
         <f>('Profit &amp; Loss'!N4-'Profit &amp; Loss'!N6)/'Profit &amp; Loss'!N4</f>
         <v/>
       </c>
+      <c r="O11" s="23">
+        <f>('Profit &amp; Loss'!O4-'Profit &amp; Loss'!O6)/'Profit &amp; Loss'!O4</f>
+        <v/>
+      </c>
+      <c r="P11" s="23">
+        <f>('Profit &amp; Loss'!P4-'Profit &amp; Loss'!P6)/'Profit &amp; Loss'!P4</f>
+        <v/>
+      </c>
+      <c r="Q11" s="23">
+        <f>('Profit &amp; Loss'!Q4-'Profit &amp; Loss'!Q6)/'Profit &amp; Loss'!Q4</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
@@ -8129,6 +8906,18 @@
         <f>'Profit &amp; Loss'!N10/'Profit &amp; Loss'!N4</f>
         <v/>
       </c>
+      <c r="O12" s="23">
+        <f>'Profit &amp; Loss'!O10/'Profit &amp; Loss'!O4</f>
+        <v/>
+      </c>
+      <c r="P12" s="23">
+        <f>'Profit &amp; Loss'!P10/'Profit &amp; Loss'!P4</f>
+        <v/>
+      </c>
+      <c r="Q12" s="23">
+        <f>'Profit &amp; Loss'!Q10/'Profit &amp; Loss'!Q4</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
@@ -8188,6 +8977,18 @@
         <f>'Profit &amp; Loss'!N13/'Profit &amp; Loss'!N4</f>
         <v/>
       </c>
+      <c r="O13" s="23">
+        <f>'Profit &amp; Loss'!O13/'Profit &amp; Loss'!O4</f>
+        <v/>
+      </c>
+      <c r="P13" s="23">
+        <f>'Profit &amp; Loss'!P13/'Profit &amp; Loss'!P4</f>
+        <v/>
+      </c>
+      <c r="Q13" s="23">
+        <f>'Profit &amp; Loss'!Q13/'Profit &amp; Loss'!Q4</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
@@ -8245,6 +9046,18 @@
       </c>
       <c r="N14" s="23">
         <f>'Profit &amp; Loss'!N21/'Profit &amp; Loss'!N4</f>
+        <v/>
+      </c>
+      <c r="O14" s="23">
+        <f>'Profit &amp; Loss'!O21/'Profit &amp; Loss'!O4</f>
+        <v/>
+      </c>
+      <c r="P14" s="23">
+        <f>'Profit &amp; Loss'!P21/'Profit &amp; Loss'!P4</f>
+        <v/>
+      </c>
+      <c r="Q14" s="23">
+        <f>'Profit &amp; Loss'!Q21/'Profit &amp; Loss'!Q4</f>
         <v/>
       </c>
     </row>
@@ -8267,6 +9080,9 @@
       <c r="L16" s="19" t="n"/>
       <c r="M16" s="19" t="n"/>
       <c r="N16" s="19" t="n"/>
+      <c r="O16" s="19" t="n"/>
+      <c r="P16" s="19" t="n"/>
+      <c r="Q16" s="19" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
@@ -8326,6 +9142,18 @@
         <f>'Profit &amp; Loss'!N21/((('Balance Sheet'!N16+'Balance Sheet'!N17)+('Balance Sheet'!M16+'Balance Sheet'!M17))/2)</f>
         <v/>
       </c>
+      <c r="O17" s="23">
+        <f>'Profit &amp; Loss'!O21/((('Balance Sheet'!O16+'Balance Sheet'!O17)+('Balance Sheet'!N16+'Balance Sheet'!N17))/2)</f>
+        <v/>
+      </c>
+      <c r="P17" s="23">
+        <f>'Profit &amp; Loss'!P21/((('Balance Sheet'!P16+'Balance Sheet'!P17)+('Balance Sheet'!O16+'Balance Sheet'!O17))/2)</f>
+        <v/>
+      </c>
+      <c r="Q17" s="23">
+        <f>'Profit &amp; Loss'!Q21/((('Balance Sheet'!Q16+'Balance Sheet'!Q17)+('Balance Sheet'!P16+'Balance Sheet'!P17))/2)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
@@ -8385,6 +9213,18 @@
         <f>'Profit &amp; Loss'!N13/((('Balance Sheet'!N16+'Balance Sheet'!N17+'Balance Sheet'!N18)+('Balance Sheet'!M16+'Balance Sheet'!M17+'Balance Sheet'!M18))/2)</f>
         <v/>
       </c>
+      <c r="O18" s="23">
+        <f>'Profit &amp; Loss'!O13/((('Balance Sheet'!O16+'Balance Sheet'!O17+'Balance Sheet'!O18)+('Balance Sheet'!N16+'Balance Sheet'!N17+'Balance Sheet'!N18))/2)</f>
+        <v/>
+      </c>
+      <c r="P18" s="23">
+        <f>'Profit &amp; Loss'!P13/((('Balance Sheet'!P16+'Balance Sheet'!P17+'Balance Sheet'!P18)+('Balance Sheet'!O16+'Balance Sheet'!O17+'Balance Sheet'!O18))/2)</f>
+        <v/>
+      </c>
+      <c r="Q18" s="23">
+        <f>'Profit &amp; Loss'!Q13/((('Balance Sheet'!Q16+'Balance Sheet'!Q17+'Balance Sheet'!Q18)+('Balance Sheet'!P16+'Balance Sheet'!P17+'Balance Sheet'!P18))/2)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
@@ -8442,6 +9282,18 @@
       </c>
       <c r="N19" s="23">
         <f>'Profit &amp; Loss'!N13*(1-'Profit &amp; Loss'!N20)/((('Balance Sheet'!N16+'Balance Sheet'!N17+'Balance Sheet'!N18-'Balance Sheet'!N11)+('Balance Sheet'!M16+'Balance Sheet'!M17+'Balance Sheet'!M18-'Balance Sheet'!M11))/2)</f>
+        <v/>
+      </c>
+      <c r="O19" s="23">
+        <f>'Profit &amp; Loss'!O13*(1-'Profit &amp; Loss'!O20)/((('Balance Sheet'!O16+'Balance Sheet'!O17+'Balance Sheet'!O18-'Balance Sheet'!O11)+('Balance Sheet'!N16+'Balance Sheet'!N17+'Balance Sheet'!N18-'Balance Sheet'!N11))/2)</f>
+        <v/>
+      </c>
+      <c r="P19" s="23">
+        <f>'Profit &amp; Loss'!P13*(1-'Profit &amp; Loss'!P20)/((('Balance Sheet'!P16+'Balance Sheet'!P17+'Balance Sheet'!P18-'Balance Sheet'!P11)+('Balance Sheet'!O16+'Balance Sheet'!O17+'Balance Sheet'!O18-'Balance Sheet'!O11))/2)</f>
+        <v/>
+      </c>
+      <c r="Q19" s="23">
+        <f>'Profit &amp; Loss'!Q13*(1-'Profit &amp; Loss'!Q20)/((('Balance Sheet'!Q16+'Balance Sheet'!Q17+'Balance Sheet'!Q18-'Balance Sheet'!Q11)+('Balance Sheet'!P16+'Balance Sheet'!P17+'Balance Sheet'!P18-'Balance Sheet'!P11))/2)</f>
         <v/>
       </c>
     </row>
@@ -8464,6 +9316,9 @@
       <c r="L21" s="19" t="n"/>
       <c r="M21" s="19" t="n"/>
       <c r="N21" s="19" t="n"/>
+      <c r="O21" s="19" t="n"/>
+      <c r="P21" s="19" t="n"/>
+      <c r="Q21" s="19" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
@@ -8523,6 +9378,18 @@
         <f>'Profit &amp; Loss'!N4/(('Balance Sheet'!N13+'Balance Sheet'!M13)/2)</f>
         <v/>
       </c>
+      <c r="O22" s="36">
+        <f>'Profit &amp; Loss'!O4/(('Balance Sheet'!O13+'Balance Sheet'!N13)/2)</f>
+        <v/>
+      </c>
+      <c r="P22" s="36">
+        <f>'Profit &amp; Loss'!P4/(('Balance Sheet'!P13+'Balance Sheet'!O13)/2)</f>
+        <v/>
+      </c>
+      <c r="Q22" s="36">
+        <f>'Profit &amp; Loss'!Q4/(('Balance Sheet'!Q13+'Balance Sheet'!P13)/2)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
@@ -8582,6 +9449,18 @@
         <f>'Working Capital Schedule'!N15</f>
         <v/>
       </c>
+      <c r="O23" s="28">
+        <f>'Working Capital Schedule'!O15</f>
+        <v/>
+      </c>
+      <c r="P23" s="28">
+        <f>'Working Capital Schedule'!P15</f>
+        <v/>
+      </c>
+      <c r="Q23" s="28">
+        <f>'Working Capital Schedule'!Q15</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
@@ -8641,6 +9520,18 @@
         <f>'Working Capital Schedule'!N14</f>
         <v/>
       </c>
+      <c r="O24" s="28">
+        <f>'Working Capital Schedule'!O14</f>
+        <v/>
+      </c>
+      <c r="P24" s="28">
+        <f>'Working Capital Schedule'!P14</f>
+        <v/>
+      </c>
+      <c r="Q24" s="28">
+        <f>'Working Capital Schedule'!Q14</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
@@ -8700,6 +9591,18 @@
         <f>'Working Capital Schedule'!N16</f>
         <v/>
       </c>
+      <c r="O25" s="28">
+        <f>'Working Capital Schedule'!O16</f>
+        <v/>
+      </c>
+      <c r="P25" s="28">
+        <f>'Working Capital Schedule'!P16</f>
+        <v/>
+      </c>
+      <c r="Q25" s="28">
+        <f>'Working Capital Schedule'!Q16</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
@@ -8757,6 +9660,18 @@
       </c>
       <c r="N26" s="28">
         <f>'Working Capital Schedule'!N17</f>
+        <v/>
+      </c>
+      <c r="O26" s="28">
+        <f>'Working Capital Schedule'!O17</f>
+        <v/>
+      </c>
+      <c r="P26" s="28">
+        <f>'Working Capital Schedule'!P17</f>
+        <v/>
+      </c>
+      <c r="Q26" s="28">
+        <f>'Working Capital Schedule'!Q17</f>
         <v/>
       </c>
     </row>
@@ -8779,6 +9694,9 @@
       <c r="L28" s="19" t="n"/>
       <c r="M28" s="19" t="n"/>
       <c r="N28" s="19" t="n"/>
+      <c r="O28" s="19" t="n"/>
+      <c r="P28" s="19" t="n"/>
+      <c r="Q28" s="19" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
@@ -8838,6 +9756,18 @@
         <f>'Balance Sheet'!N18/('Balance Sheet'!N16+'Balance Sheet'!N17)</f>
         <v/>
       </c>
+      <c r="O29" s="36">
+        <f>'Balance Sheet'!O18/('Balance Sheet'!O16+'Balance Sheet'!O17)</f>
+        <v/>
+      </c>
+      <c r="P29" s="36">
+        <f>'Balance Sheet'!P18/('Balance Sheet'!P16+'Balance Sheet'!P17)</f>
+        <v/>
+      </c>
+      <c r="Q29" s="36">
+        <f>'Balance Sheet'!Q18/('Balance Sheet'!Q16+'Balance Sheet'!Q17)</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
@@ -8897,6 +9827,18 @@
         <f>'Working Schedules'!N28/'Profit &amp; Loss'!N10</f>
         <v/>
       </c>
+      <c r="O30" s="36">
+        <f>'Working Schedules'!O28/'Profit &amp; Loss'!O10</f>
+        <v/>
+      </c>
+      <c r="P30" s="36">
+        <f>'Working Schedules'!P28/'Profit &amp; Loss'!P10</f>
+        <v/>
+      </c>
+      <c r="Q30" s="36">
+        <f>'Working Schedules'!Q28/'Profit &amp; Loss'!Q10</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
@@ -8954,6 +9896,18 @@
       </c>
       <c r="N31" s="36">
         <f>IF('Profit &amp; Loss'!N15=0,"",'Profit &amp; Loss'!N13/'Profit &amp; Loss'!N15)</f>
+        <v/>
+      </c>
+      <c r="O31" s="36">
+        <f>IF('Profit &amp; Loss'!O15=0,"",'Profit &amp; Loss'!O13/'Profit &amp; Loss'!O15)</f>
+        <v/>
+      </c>
+      <c r="P31" s="36">
+        <f>IF('Profit &amp; Loss'!P15=0,"",'Profit &amp; Loss'!P13/'Profit &amp; Loss'!P15)</f>
+        <v/>
+      </c>
+      <c r="Q31" s="36">
+        <f>IF('Profit &amp; Loss'!Q15=0,"",'Profit &amp; Loss'!Q13/'Profit &amp; Loss'!Q15)</f>
         <v/>
       </c>
     </row>
@@ -8968,7 +9922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:Q22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -8985,6 +9939,9 @@
     <col width="12.5" customWidth="1" min="12" max="12"/>
     <col width="12.5" customWidth="1" min="13" max="13"/>
     <col width="12.5" customWidth="1" min="14" max="14"/>
+    <col width="12.5" customWidth="1" min="15" max="15"/>
+    <col width="12.5" customWidth="1" min="16" max="16"/>
+    <col width="12.5" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -9006,6 +9963,9 @@
       <c r="L1" s="2" t="n"/>
       <c r="M1" s="2" t="n"/>
       <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -9085,6 +10045,21 @@
           <t>FY2033E</t>
         </is>
       </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>FY2034E</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>FY2035E</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>FY2036E</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -9138,6 +10113,18 @@
         <f>Assumptions!N44</f>
         <v/>
       </c>
+      <c r="O4" s="22">
+        <f>Assumptions!O44</f>
+        <v/>
+      </c>
+      <c r="P4" s="22">
+        <f>Assumptions!P44</f>
+        <v/>
+      </c>
+      <c r="Q4" s="22">
+        <f>Assumptions!Q44</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -9193,6 +10180,18 @@
         <f>IF(Assumptions!M44=0,"",Assumptions!N44/Assumptions!M44-1)</f>
         <v/>
       </c>
+      <c r="O5" s="10">
+        <f>IF(Assumptions!N44=0,"",Assumptions!O44/Assumptions!N44-1)</f>
+        <v/>
+      </c>
+      <c r="P5" s="10">
+        <f>IF(Assumptions!O44=0,"",Assumptions!P44/Assumptions!O44-1)</f>
+        <v/>
+      </c>
+      <c r="Q5" s="10">
+        <f>IF(Assumptions!P44=0,"",Assumptions!Q44/Assumptions!P44-1)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
@@ -9246,6 +10245,18 @@
         <f>N4*Assumptions!N6</f>
         <v/>
       </c>
+      <c r="O6" s="13">
+        <f>O4*Assumptions!O6</f>
+        <v/>
+      </c>
+      <c r="P6" s="13">
+        <f>P4*Assumptions!P6</f>
+        <v/>
+      </c>
+      <c r="Q6" s="13">
+        <f>Q4*Assumptions!Q6</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
@@ -9299,6 +10310,18 @@
         <f>N4*Assumptions!N7</f>
         <v/>
       </c>
+      <c r="O7" s="13">
+        <f>O4*Assumptions!O7</f>
+        <v/>
+      </c>
+      <c r="P7" s="13">
+        <f>P4*Assumptions!P7</f>
+        <v/>
+      </c>
+      <c r="Q7" s="13">
+        <f>Q4*Assumptions!Q7</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
@@ -9352,6 +10375,18 @@
         <f>N4*(Assumptions!N8-Assumptions!$B$58)</f>
         <v/>
       </c>
+      <c r="O8" s="13">
+        <f>O4*(Assumptions!O8-Assumptions!$B$58)</f>
+        <v/>
+      </c>
+      <c r="P8" s="13">
+        <f>P4*(Assumptions!P8-Assumptions!$B$58)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="13">
+        <f>Q4*(Assumptions!Q8-Assumptions!$B$58)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -9411,6 +10446,18 @@
         <f>SUM(N6:N8)</f>
         <v/>
       </c>
+      <c r="O9" s="14">
+        <f>SUM(O6:O8)</f>
+        <v/>
+      </c>
+      <c r="P9" s="14">
+        <f>SUM(P6:P8)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="14">
+        <f>SUM(Q6:Q8)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -9470,6 +10517,18 @@
         <f>N4-N9</f>
         <v/>
       </c>
+      <c r="O10" s="15">
+        <f>O4-O9</f>
+        <v/>
+      </c>
+      <c r="P10" s="15">
+        <f>P4-P9</f>
+        <v/>
+      </c>
+      <c r="Q10" s="15">
+        <f>Q4-Q9</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -9529,6 +10588,18 @@
         <f>IF(N4=0,"",N10/N4)</f>
         <v/>
       </c>
+      <c r="O11" s="10">
+        <f>IF(O4=0,"",O10/O4)</f>
+        <v/>
+      </c>
+      <c r="P11" s="10">
+        <f>IF(P4=0,"",P10/P4)</f>
+        <v/>
+      </c>
+      <c r="Q11" s="10">
+        <f>IF(Q4=0,"",Q10/Q4)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
@@ -9582,6 +10653,18 @@
         <f>'Working Schedules'!N6</f>
         <v/>
       </c>
+      <c r="O12" s="16">
+        <f>'Working Schedules'!O6</f>
+        <v/>
+      </c>
+      <c r="P12" s="16">
+        <f>'Working Schedules'!P6</f>
+        <v/>
+      </c>
+      <c r="Q12" s="16">
+        <f>'Working Schedules'!Q6</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -9641,6 +10724,18 @@
         <f>N10-N12</f>
         <v/>
       </c>
+      <c r="O13" s="77">
+        <f>O10-O12</f>
+        <v/>
+      </c>
+      <c r="P13" s="77">
+        <f>P10-P12</f>
+        <v/>
+      </c>
+      <c r="Q13" s="77">
+        <f>Q10-Q12</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
@@ -9694,6 +10789,18 @@
         <f>N4*Assumptions!N9</f>
         <v/>
       </c>
+      <c r="O14" s="13">
+        <f>O4*Assumptions!O9</f>
+        <v/>
+      </c>
+      <c r="P14" s="13">
+        <f>P4*Assumptions!P9</f>
+        <v/>
+      </c>
+      <c r="Q14" s="13">
+        <f>Q4*Assumptions!Q9</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
@@ -9747,6 +10854,18 @@
         <f>'Working Schedules'!N13</f>
         <v/>
       </c>
+      <c r="O15" s="16">
+        <f>'Working Schedules'!O13</f>
+        <v/>
+      </c>
+      <c r="P15" s="16">
+        <f>'Working Schedules'!P13</f>
+        <v/>
+      </c>
+      <c r="Q15" s="16">
+        <f>'Working Schedules'!Q13</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
@@ -9806,6 +10925,18 @@
         <f>N13+N14-N15</f>
         <v/>
       </c>
+      <c r="O16" s="13">
+        <f>O13+O14-O15</f>
+        <v/>
+      </c>
+      <c r="P16" s="13">
+        <f>P13+P14-P15</f>
+        <v/>
+      </c>
+      <c r="Q16" s="13">
+        <f>Q13+Q14-Q15</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
@@ -9852,6 +10983,15 @@
       <c r="N17" s="12" t="n">
         <v>0</v>
       </c>
+      <c r="O17" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -9911,6 +11051,18 @@
         <f>N16+N17</f>
         <v/>
       </c>
+      <c r="O18" s="14">
+        <f>O16+O17</f>
+        <v/>
+      </c>
+      <c r="P18" s="14">
+        <f>P16+P17</f>
+        <v/>
+      </c>
+      <c r="Q18" s="14">
+        <f>Q16+Q17</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
@@ -9964,6 +11116,18 @@
         <f>N18*Assumptions!N12</f>
         <v/>
       </c>
+      <c r="O19" s="13">
+        <f>O18*Assumptions!O12</f>
+        <v/>
+      </c>
+      <c r="P19" s="13">
+        <f>P18*Assumptions!P12</f>
+        <v/>
+      </c>
+      <c r="Q19" s="13">
+        <f>Q18*Assumptions!Q12</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
@@ -10023,6 +11187,18 @@
         <f>IF(N18=0,"",N19/N18)</f>
         <v/>
       </c>
+      <c r="O20" s="10">
+        <f>IF(O18=0,"",O19/O18)</f>
+        <v/>
+      </c>
+      <c r="P20" s="10">
+        <f>IF(P18=0,"",P19/P18)</f>
+        <v/>
+      </c>
+      <c r="Q20" s="10">
+        <f>IF(Q18=0,"",Q19/Q18)</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -10076,6 +11252,18 @@
         <f>N18-N19</f>
         <v/>
       </c>
+      <c r="O21" s="15">
+        <f>O18-O19</f>
+        <v/>
+      </c>
+      <c r="P21" s="15">
+        <f>P18-P19</f>
+        <v/>
+      </c>
+      <c r="Q21" s="15">
+        <f>Q18-Q19</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
@@ -10133,6 +11321,18 @@
       </c>
       <c r="N22" s="13">
         <f>IF('Working Schedules'!N23=0,"",N21/'Working Schedules'!N23)</f>
+        <v/>
+      </c>
+      <c r="O22" s="13">
+        <f>IF('Working Schedules'!O23=0,"",O21/'Working Schedules'!O23)</f>
+        <v/>
+      </c>
+      <c r="P22" s="13">
+        <f>IF('Working Schedules'!P23=0,"",P21/'Working Schedules'!P23)</f>
+        <v/>
+      </c>
+      <c r="Q22" s="13">
+        <f>IF('Working Schedules'!Q23=0,"",Q21/'Working Schedules'!Q23)</f>
         <v/>
       </c>
     </row>
@@ -10147,7 +11347,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:Q25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -10164,6 +11364,9 @@
     <col width="12.5" customWidth="1" min="12" max="12"/>
     <col width="12.5" customWidth="1" min="13" max="13"/>
     <col width="12.5" customWidth="1" min="14" max="14"/>
+    <col width="12.5" customWidth="1" min="15" max="15"/>
+    <col width="12.5" customWidth="1" min="16" max="16"/>
+    <col width="12.5" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -10185,6 +11388,9 @@
       <c r="L1" s="2" t="n"/>
       <c r="M1" s="2" t="n"/>
       <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -10262,6 +11468,21 @@
       <c r="N3" s="5" t="inlineStr">
         <is>
           <t>FY2033E</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>FY2034E</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>FY2035E</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>FY2036E</t>
         </is>
       </c>
     </row>
@@ -10284,6 +11505,9 @@
       <c r="L4" s="19" t="n"/>
       <c r="M4" s="19" t="n"/>
       <c r="N4" s="19" t="n"/>
+      <c r="O4" s="19" t="n"/>
+      <c r="P4" s="19" t="n"/>
+      <c r="Q4" s="19" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -10337,6 +11561,18 @@
         <f>'Working Schedules'!N8</f>
         <v/>
       </c>
+      <c r="O5" s="16">
+        <f>'Working Schedules'!O8</f>
+        <v/>
+      </c>
+      <c r="P5" s="16">
+        <f>'Working Schedules'!P8</f>
+        <v/>
+      </c>
+      <c r="Q5" s="16">
+        <f>'Working Schedules'!Q8</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
@@ -10390,6 +11626,18 @@
         <f>M6</f>
         <v/>
       </c>
+      <c r="O6" s="13">
+        <f>N6</f>
+        <v/>
+      </c>
+      <c r="P6" s="13">
+        <f>O6</f>
+        <v/>
+      </c>
+      <c r="Q6" s="13">
+        <f>P6</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
@@ -10443,6 +11691,18 @@
         <f>M7</f>
         <v/>
       </c>
+      <c r="O7" s="13">
+        <f>N7</f>
+        <v/>
+      </c>
+      <c r="P7" s="13">
+        <f>O7</f>
+        <v/>
+      </c>
+      <c r="Q7" s="13">
+        <f>P7</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
@@ -10496,6 +11756,18 @@
         <f>M8</f>
         <v/>
       </c>
+      <c r="O8" s="13">
+        <f>N8</f>
+        <v/>
+      </c>
+      <c r="P8" s="13">
+        <f>O8</f>
+        <v/>
+      </c>
+      <c r="Q8" s="13">
+        <f>P8</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
@@ -10549,6 +11821,18 @@
         <f>'Working Capital Schedule'!N7</f>
         <v/>
       </c>
+      <c r="O9" s="16">
+        <f>'Working Capital Schedule'!O7</f>
+        <v/>
+      </c>
+      <c r="P9" s="16">
+        <f>'Working Capital Schedule'!P7</f>
+        <v/>
+      </c>
+      <c r="Q9" s="16">
+        <f>'Working Capital Schedule'!Q7</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
@@ -10602,6 +11886,18 @@
         <f>'Working Capital Schedule'!N6</f>
         <v/>
       </c>
+      <c r="O10" s="16">
+        <f>'Working Capital Schedule'!O6</f>
+        <v/>
+      </c>
+      <c r="P10" s="16">
+        <f>'Working Capital Schedule'!P6</f>
+        <v/>
+      </c>
+      <c r="Q10" s="16">
+        <f>'Working Capital Schedule'!Q6</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
@@ -10655,6 +11951,18 @@
         <f>'Cash Flow Statement'!N21</f>
         <v/>
       </c>
+      <c r="O11" s="16">
+        <f>'Cash Flow Statement'!O21</f>
+        <v/>
+      </c>
+      <c r="P11" s="16">
+        <f>'Cash Flow Statement'!P21</f>
+        <v/>
+      </c>
+      <c r="Q11" s="16">
+        <f>'Cash Flow Statement'!Q21</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
@@ -10708,6 +12016,18 @@
         <f>'Working Capital Schedule'!N8</f>
         <v/>
       </c>
+      <c r="O12" s="16">
+        <f>'Working Capital Schedule'!O8</f>
+        <v/>
+      </c>
+      <c r="P12" s="16">
+        <f>'Working Capital Schedule'!P8</f>
+        <v/>
+      </c>
+      <c r="Q12" s="16">
+        <f>'Working Capital Schedule'!Q8</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -10765,6 +12085,18 @@
       </c>
       <c r="N13" s="20">
         <f>SUM(N5:N12)</f>
+        <v/>
+      </c>
+      <c r="O13" s="20">
+        <f>SUM(O5:O12)</f>
+        <v/>
+      </c>
+      <c r="P13" s="20">
+        <f>SUM(P5:P12)</f>
+        <v/>
+      </c>
+      <c r="Q13" s="20">
+        <f>SUM(Q5:Q12)</f>
         <v/>
       </c>
     </row>
@@ -10787,6 +12119,9 @@
       <c r="L15" s="19" t="n"/>
       <c r="M15" s="19" t="n"/>
       <c r="N15" s="19" t="n"/>
+      <c r="O15" s="19" t="n"/>
+      <c r="P15" s="19" t="n"/>
+      <c r="Q15" s="19" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
@@ -10840,6 +12175,18 @@
         <f>M16</f>
         <v/>
       </c>
+      <c r="O16" s="13">
+        <f>N16</f>
+        <v/>
+      </c>
+      <c r="P16" s="13">
+        <f>O16</f>
+        <v/>
+      </c>
+      <c r="Q16" s="13">
+        <f>P16</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
@@ -10893,6 +12240,18 @@
         <f>'Working Schedules'!N21</f>
         <v/>
       </c>
+      <c r="O17" s="16">
+        <f>'Working Schedules'!O21</f>
+        <v/>
+      </c>
+      <c r="P17" s="16">
+        <f>'Working Schedules'!P21</f>
+        <v/>
+      </c>
+      <c r="Q17" s="16">
+        <f>'Working Schedules'!Q21</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
@@ -10946,6 +12305,18 @@
         <f>'Working Schedules'!N12</f>
         <v/>
       </c>
+      <c r="O18" s="16">
+        <f>'Working Schedules'!O12</f>
+        <v/>
+      </c>
+      <c r="P18" s="16">
+        <f>'Working Schedules'!P12</f>
+        <v/>
+      </c>
+      <c r="Q18" s="16">
+        <f>'Working Schedules'!Q12</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
@@ -10999,6 +12370,18 @@
         <f>M19</f>
         <v/>
       </c>
+      <c r="O19" s="13">
+        <f>N19</f>
+        <v/>
+      </c>
+      <c r="P19" s="13">
+        <f>O19</f>
+        <v/>
+      </c>
+      <c r="Q19" s="13">
+        <f>P19</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
@@ -11052,6 +12435,18 @@
         <f>M20</f>
         <v/>
       </c>
+      <c r="O20" s="13">
+        <f>N20</f>
+        <v/>
+      </c>
+      <c r="P20" s="13">
+        <f>O20</f>
+        <v/>
+      </c>
+      <c r="Q20" s="13">
+        <f>P20</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
@@ -11105,6 +12500,18 @@
         <f>'Working Capital Schedule'!N9</f>
         <v/>
       </c>
+      <c r="O21" s="16">
+        <f>'Working Capital Schedule'!O9</f>
+        <v/>
+      </c>
+      <c r="P21" s="16">
+        <f>'Working Capital Schedule'!P9</f>
+        <v/>
+      </c>
+      <c r="Q21" s="16">
+        <f>'Working Capital Schedule'!Q9</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
@@ -11158,6 +12565,18 @@
         <f>'Working Capital Schedule'!N10</f>
         <v/>
       </c>
+      <c r="O22" s="16">
+        <f>'Working Capital Schedule'!O10</f>
+        <v/>
+      </c>
+      <c r="P22" s="16">
+        <f>'Working Capital Schedule'!P10</f>
+        <v/>
+      </c>
+      <c r="Q22" s="16">
+        <f>'Working Capital Schedule'!Q10</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -11217,6 +12636,18 @@
         <f>SUM(N16:N22)</f>
         <v/>
       </c>
+      <c r="O23" s="20">
+        <f>SUM(O16:O22)</f>
+        <v/>
+      </c>
+      <c r="P23" s="20">
+        <f>SUM(P16:P22)</f>
+        <v/>
+      </c>
+      <c r="Q23" s="20">
+        <f>SUM(Q16:Q22)</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
@@ -11274,6 +12705,18 @@
       </c>
       <c r="N25" s="21">
         <f>N13-N23</f>
+        <v/>
+      </c>
+      <c r="O25" s="21">
+        <f>O13-O23</f>
+        <v/>
+      </c>
+      <c r="P25" s="21">
+        <f>P13-P23</f>
+        <v/>
+      </c>
+      <c r="Q25" s="21">
+        <f>Q13-Q23</f>
         <v/>
       </c>
     </row>
@@ -11288,7 +12731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -11305,6 +12748,9 @@
     <col width="12.5" customWidth="1" min="12" max="12"/>
     <col width="12.5" customWidth="1" min="13" max="13"/>
     <col width="12.5" customWidth="1" min="14" max="14"/>
+    <col width="12.5" customWidth="1" min="15" max="15"/>
+    <col width="12.5" customWidth="1" min="16" max="16"/>
+    <col width="12.5" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -11326,6 +12772,9 @@
       <c r="L1" s="2" t="n"/>
       <c r="M1" s="2" t="n"/>
       <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -11405,6 +12854,21 @@
           <t>FY2033E</t>
         </is>
       </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>FY2034E</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>FY2035E</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>FY2036E</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -11440,6 +12904,18 @@
         <f>'Profit &amp; Loss'!N21</f>
         <v/>
       </c>
+      <c r="O4" s="16">
+        <f>'Profit &amp; Loss'!O21</f>
+        <v/>
+      </c>
+      <c r="P4" s="16">
+        <f>'Profit &amp; Loss'!P21</f>
+        <v/>
+      </c>
+      <c r="Q4" s="16">
+        <f>'Profit &amp; Loss'!Q21</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -11475,6 +12951,18 @@
         <f>'Profit &amp; Loss'!N12</f>
         <v/>
       </c>
+      <c r="O5" s="16">
+        <f>'Profit &amp; Loss'!O12</f>
+        <v/>
+      </c>
+      <c r="P5" s="16">
+        <f>'Profit &amp; Loss'!P12</f>
+        <v/>
+      </c>
+      <c r="Q5" s="16">
+        <f>'Profit &amp; Loss'!Q12</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
@@ -11510,6 +12998,18 @@
         <f>'Profit &amp; Loss'!N15</f>
         <v/>
       </c>
+      <c r="O6" s="16">
+        <f>'Profit &amp; Loss'!O15</f>
+        <v/>
+      </c>
+      <c r="P6" s="16">
+        <f>'Profit &amp; Loss'!P15</f>
+        <v/>
+      </c>
+      <c r="Q6" s="16">
+        <f>'Profit &amp; Loss'!Q15</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
@@ -11545,6 +13045,18 @@
         <f>'Working Capital Schedule'!N12</f>
         <v/>
       </c>
+      <c r="O7" s="16">
+        <f>'Working Capital Schedule'!O12</f>
+        <v/>
+      </c>
+      <c r="P7" s="16">
+        <f>'Working Capital Schedule'!P12</f>
+        <v/>
+      </c>
+      <c r="Q7" s="16">
+        <f>'Working Capital Schedule'!Q12</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -11598,6 +13110,18 @@
         <f>N4+N5+N6-N7</f>
         <v/>
       </c>
+      <c r="O8" s="15">
+        <f>O4+O5+O6-O7</f>
+        <v/>
+      </c>
+      <c r="P8" s="15">
+        <f>P4+P5+P6-P7</f>
+        <v/>
+      </c>
+      <c r="Q8" s="15">
+        <f>Q4+Q5+Q6-Q7</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
@@ -11651,6 +13175,18 @@
         <f>Assumptions!N11</f>
         <v/>
       </c>
+      <c r="O10" s="16">
+        <f>Assumptions!O11</f>
+        <v/>
+      </c>
+      <c r="P10" s="16">
+        <f>Assumptions!P11</f>
+        <v/>
+      </c>
+      <c r="Q10" s="16">
+        <f>Assumptions!Q11</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -11704,6 +13240,18 @@
         <f>-N10</f>
         <v/>
       </c>
+      <c r="O11" s="15">
+        <f>-O10</f>
+        <v/>
+      </c>
+      <c r="P11" s="15">
+        <f>-P10</f>
+        <v/>
+      </c>
+      <c r="Q11" s="15">
+        <f>-Q10</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
@@ -11739,6 +13287,18 @@
         <f>'Working Schedules'!N12-'Working Schedules'!N11</f>
         <v/>
       </c>
+      <c r="O13" s="13">
+        <f>'Working Schedules'!O12-'Working Schedules'!O11</f>
+        <v/>
+      </c>
+      <c r="P13" s="13">
+        <f>'Working Schedules'!P12-'Working Schedules'!P11</f>
+        <v/>
+      </c>
+      <c r="Q13" s="13">
+        <f>'Working Schedules'!Q12-'Working Schedules'!Q11</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
@@ -11774,6 +13334,18 @@
         <f>-'Profit &amp; Loss'!N15</f>
         <v/>
       </c>
+      <c r="O14" s="13">
+        <f>-'Profit &amp; Loss'!O15</f>
+        <v/>
+      </c>
+      <c r="P14" s="13">
+        <f>-'Profit &amp; Loss'!P15</f>
+        <v/>
+      </c>
+      <c r="Q14" s="13">
+        <f>-'Profit &amp; Loss'!Q15</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
@@ -11809,6 +13381,18 @@
         <f>-'Working Schedules'!N19</f>
         <v/>
       </c>
+      <c r="O15" s="13">
+        <f>-'Working Schedules'!O19</f>
+        <v/>
+      </c>
+      <c r="P15" s="13">
+        <f>-'Working Schedules'!P19</f>
+        <v/>
+      </c>
+      <c r="Q15" s="13">
+        <f>-'Working Schedules'!Q19</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
@@ -11844,6 +13428,18 @@
         <f>'Working Schedules'!N20</f>
         <v/>
       </c>
+      <c r="O16" s="16">
+        <f>'Working Schedules'!O20</f>
+        <v/>
+      </c>
+      <c r="P16" s="16">
+        <f>'Working Schedules'!P20</f>
+        <v/>
+      </c>
+      <c r="Q16" s="16">
+        <f>'Working Schedules'!Q20</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -11897,6 +13493,18 @@
         <f>N13+N14+N15+N16</f>
         <v/>
       </c>
+      <c r="O17" s="15">
+        <f>O13+O14+O15+O16</f>
+        <v/>
+      </c>
+      <c r="P17" s="15">
+        <f>P13+P14+P15+P16</f>
+        <v/>
+      </c>
+      <c r="Q17" s="15">
+        <f>Q13+Q14+Q15+Q16</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -11956,6 +13564,18 @@
         <f>N8+N11+N17</f>
         <v/>
       </c>
+      <c r="O19" s="77">
+        <f>O8+O11+O17</f>
+        <v/>
+      </c>
+      <c r="P19" s="77">
+        <f>P8+P11+P17</f>
+        <v/>
+      </c>
+      <c r="Q19" s="77">
+        <f>Q8+Q11+Q17</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
@@ -11991,6 +13611,18 @@
         <f>M21</f>
         <v/>
       </c>
+      <c r="O20" s="13">
+        <f>N21</f>
+        <v/>
+      </c>
+      <c r="P20" s="13">
+        <f>O21</f>
+        <v/>
+      </c>
+      <c r="Q20" s="13">
+        <f>P21</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -12048,6 +13680,18 @@
       </c>
       <c r="N21" s="15">
         <f>N20+N19</f>
+        <v/>
+      </c>
+      <c r="O21" s="15">
+        <f>O20+O19</f>
+        <v/>
+      </c>
+      <c r="P21" s="15">
+        <f>P20+P19</f>
+        <v/>
+      </c>
+      <c r="Q21" s="15">
+        <f>Q20+Q19</f>
         <v/>
       </c>
     </row>
@@ -12062,7 +13706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N61"/>
+  <dimension ref="A1:Q61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -12079,6 +13723,9 @@
     <col width="12.5" customWidth="1" min="12" max="12"/>
     <col width="12.5" customWidth="1" min="13" max="13"/>
     <col width="12.5" customWidth="1" min="14" max="14"/>
+    <col width="12.5" customWidth="1" min="15" max="15"/>
+    <col width="12.5" customWidth="1" min="16" max="16"/>
+    <col width="12.5" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -12100,6 +13747,9 @@
       <c r="L1" s="2" t="n"/>
       <c r="M1" s="2" t="n"/>
       <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -12177,6 +13827,21 @@
       <c r="N3" s="5" t="inlineStr">
         <is>
           <t>FY2033E</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>FY2034E</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>FY2035E</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>FY2036E</t>
         </is>
       </c>
     </row>
@@ -12235,6 +13900,18 @@
         <f>IF(M44=0,"",N44/M44-1)</f>
         <v/>
       </c>
+      <c r="O5" s="79">
+        <f>IF(N44=0,"",O44/N44-1)</f>
+        <v/>
+      </c>
+      <c r="P5" s="79">
+        <f>IF(O44=0,"",P44/O44-1)</f>
+        <v/>
+      </c>
+      <c r="Q5" s="79">
+        <f>IF(P44=0,"",Q44/P44-1)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
@@ -12287,6 +13964,15 @@
       <c r="N6" s="76" t="n">
         <v>0.41</v>
       </c>
+      <c r="O6" s="76" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="P6" s="76" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="Q6" s="76" t="n">
+        <v>0.41</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
@@ -12339,6 +14025,15 @@
       <c r="N7" s="76" t="n">
         <v>0.11</v>
       </c>
+      <c r="O7" s="76" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="P7" s="76" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="Q7" s="76" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
@@ -12391,6 +14086,15 @@
       <c r="N8" s="76" t="n">
         <v>0.185</v>
       </c>
+      <c r="O8" s="76" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="P8" s="76" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="Q8" s="76" t="n">
+        <v>0.185</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
@@ -12441,6 +14145,15 @@
         <v>0.015</v>
       </c>
       <c r="N9" s="76" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="O9" s="76" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="P9" s="76" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="Q9" s="76" t="n">
         <v>0.015</v>
       </c>
     </row>
@@ -12492,6 +14205,15 @@
       <c r="N10" s="76" t="n">
         <v>0.06</v>
       </c>
+      <c r="O10" s="76" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="P10" s="76" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="Q10" s="76" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
@@ -12538,6 +14260,15 @@
       <c r="N11" s="26" t="n">
         <v>450</v>
       </c>
+      <c r="O11" s="26" t="n">
+        <v>440</v>
+      </c>
+      <c r="P11" s="26" t="n">
+        <v>430</v>
+      </c>
+      <c r="Q11" s="26" t="n">
+        <v>420</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
@@ -12588,6 +14319,15 @@
         <v>0.25</v>
       </c>
       <c r="N12" s="76" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="O12" s="76" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="P12" s="76" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Q12" s="76" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -12624,6 +14364,15 @@
       <c r="N13" s="76" t="n">
         <v>0.15</v>
       </c>
+      <c r="O13" s="76" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P13" s="76" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q13" s="76" t="n">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
@@ -12676,6 +14425,15 @@
       <c r="N14" s="29" t="n">
         <v>85</v>
       </c>
+      <c r="O14" s="29" t="n">
+        <v>85</v>
+      </c>
+      <c r="P14" s="29" t="n">
+        <v>85</v>
+      </c>
+      <c r="Q14" s="29" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
@@ -12728,6 +14486,15 @@
       <c r="N15" s="29" t="n">
         <v>115</v>
       </c>
+      <c r="O15" s="29" t="n">
+        <v>115</v>
+      </c>
+      <c r="P15" s="29" t="n">
+        <v>115</v>
+      </c>
+      <c r="Q15" s="29" t="n">
+        <v>115</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
@@ -12780,6 +14547,15 @@
       <c r="N16" s="29" t="n">
         <v>130</v>
       </c>
+      <c r="O16" s="29" t="n">
+        <v>130</v>
+      </c>
+      <c r="P16" s="29" t="n">
+        <v>130</v>
+      </c>
+      <c r="Q16" s="29" t="n">
+        <v>130</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
@@ -12832,6 +14608,15 @@
       <c r="N17" s="76" t="n">
         <v>0.06</v>
       </c>
+      <c r="O17" s="76" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="P17" s="76" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="Q17" s="76" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
@@ -12884,6 +14669,15 @@
       <c r="N18" s="76" t="n">
         <v>0.07000000000000001</v>
       </c>
+      <c r="O18" s="76" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="P18" s="76" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="Q18" s="76" t="n">
+        <v>0.07000000000000001</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
@@ -12935,6 +14729,15 @@
       </c>
       <c r="N19" s="26" t="n">
         <v>400</v>
+      </c>
+      <c r="O19" s="26" t="n">
+        <v>350</v>
+      </c>
+      <c r="P19" s="26" t="n">
+        <v>300</v>
+      </c>
+      <c r="Q19" s="26" t="n">
+        <v>250</v>
       </c>
     </row>
     <row r="20">
@@ -12983,6 +14786,15 @@
         <v>0.075</v>
       </c>
       <c r="N20" s="76" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="O20" s="76" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="P20" s="76" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="Q20" s="76" t="n">
         <v>0.075</v>
       </c>
     </row>
@@ -13005,6 +14817,9 @@
       <c r="L23" s="19" t="n"/>
       <c r="M23" s="19" t="n"/>
       <c r="N23" s="19" t="n"/>
+      <c r="O23" s="19" t="n"/>
+      <c r="P23" s="19" t="n"/>
+      <c r="Q23" s="19" t="n"/>
     </row>
     <row r="24" ht="42" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
@@ -13145,6 +14960,9 @@
       <c r="L40" s="19" t="n"/>
       <c r="M40" s="19" t="n"/>
       <c r="N40" s="19" t="n"/>
+      <c r="O40" s="19" t="n"/>
+      <c r="P40" s="19" t="n"/>
+      <c r="Q40" s="19" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="11" t="inlineStr">
@@ -13198,6 +15016,18 @@
         <f>M41*(1+N47+$B$57)</f>
         <v/>
       </c>
+      <c r="O41" s="13">
+        <f>N41*(1+O47+$B$57)</f>
+        <v/>
+      </c>
+      <c r="P41" s="13">
+        <f>O41*(1+P47+$B$57)</f>
+        <v/>
+      </c>
+      <c r="Q41" s="13">
+        <f>P41*(1+Q47+$B$57)</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
@@ -13251,6 +15081,18 @@
         <f>M42*(1+N48+$B$57)</f>
         <v/>
       </c>
+      <c r="O42" s="13">
+        <f>N42*(1+O48+$B$57)</f>
+        <v/>
+      </c>
+      <c r="P42" s="13">
+        <f>O42*(1+P48+$B$57)</f>
+        <v/>
+      </c>
+      <c r="Q42" s="13">
+        <f>P42*(1+Q48+$B$57)</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="11" t="inlineStr">
@@ -13310,6 +15152,18 @@
         <f>M43*(1+N49+$B$57)</f>
         <v/>
       </c>
+      <c r="O43" s="13">
+        <f>N43*(1+O49+$B$57)</f>
+        <v/>
+      </c>
+      <c r="P43" s="13">
+        <f>O43*(1+P49+$B$57)</f>
+        <v/>
+      </c>
+      <c r="Q43" s="13">
+        <f>P43*(1+Q49+$B$57)</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
@@ -13367,6 +15221,18 @@
       </c>
       <c r="N44" s="14">
         <f>SUM(N41:N43)</f>
+        <v/>
+      </c>
+      <c r="O44" s="14">
+        <f>SUM(O41:O43)</f>
+        <v/>
+      </c>
+      <c r="P44" s="14">
+        <f>SUM(P41:P43)</f>
+        <v/>
+      </c>
+      <c r="Q44" s="14">
+        <f>SUM(Q41:Q43)</f>
         <v/>
       </c>
     </row>
@@ -13389,6 +15255,9 @@
       <c r="L46" s="19" t="n"/>
       <c r="M46" s="19" t="n"/>
       <c r="N46" s="19" t="n"/>
+      <c r="O46" s="19" t="n"/>
+      <c r="P46" s="19" t="n"/>
+      <c r="Q46" s="19" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="11" t="inlineStr">
@@ -13437,6 +15306,15 @@
       <c r="N47" s="76" t="n">
         <v>0.09</v>
       </c>
+      <c r="O47" s="76" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="P47" s="76" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="Q47" s="76" t="n">
+        <v>0.08</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="11" t="inlineStr">
@@ -13485,6 +15363,15 @@
       <c r="N48" s="76" t="n">
         <v>0.12</v>
       </c>
+      <c r="O48" s="76" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="P48" s="76" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q48" s="76" t="n">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="11" t="inlineStr">
@@ -13532,6 +15419,15 @@
       </c>
       <c r="N49" s="76" t="n">
         <v>0.16</v>
+      </c>
+      <c r="O49" s="76" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P49" s="76" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="Q49" s="76" t="n">
+        <v>0.13</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1">
@@ -13562,6 +15458,9 @@
       <c r="L54" s="19" t="n"/>
       <c r="M54" s="19" t="n"/>
       <c r="N54" s="19" t="n"/>
+      <c r="O54" s="19" t="n"/>
+      <c r="P54" s="19" t="n"/>
+      <c r="Q54" s="19" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
@@ -13729,7 +15628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -13746,6 +15645,9 @@
     <col width="12.5" customWidth="1" min="12" max="12"/>
     <col width="12.5" customWidth="1" min="13" max="13"/>
     <col width="12.5" customWidth="1" min="14" max="14"/>
+    <col width="12.5" customWidth="1" min="15" max="15"/>
+    <col width="12.5" customWidth="1" min="16" max="16"/>
+    <col width="12.5" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -13767,6 +15669,9 @@
       <c r="L1" s="2" t="n"/>
       <c r="M1" s="2" t="n"/>
       <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -13846,6 +15751,21 @@
           <t>FY2033E</t>
         </is>
       </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>FY2034E</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>FY2035E</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>FY2036E</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -13905,6 +15825,18 @@
         <f>'Profit &amp; Loss'!N4</f>
         <v/>
       </c>
+      <c r="O4" s="16">
+        <f>'Profit &amp; Loss'!O4</f>
+        <v/>
+      </c>
+      <c r="P4" s="16">
+        <f>'Profit &amp; Loss'!P4</f>
+        <v/>
+      </c>
+      <c r="Q4" s="16">
+        <f>'Profit &amp; Loss'!Q4</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -13964,6 +15896,18 @@
         <f>'Profit &amp; Loss'!N6</f>
         <v/>
       </c>
+      <c r="O5" s="16">
+        <f>'Profit &amp; Loss'!O6</f>
+        <v/>
+      </c>
+      <c r="P5" s="16">
+        <f>'Profit &amp; Loss'!P6</f>
+        <v/>
+      </c>
+      <c r="Q5" s="16">
+        <f>'Profit &amp; Loss'!Q6</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
@@ -14023,6 +15967,18 @@
         <f>Assumptions!N14/365*N4</f>
         <v/>
       </c>
+      <c r="O6" s="13">
+        <f>Assumptions!O14/365*O4</f>
+        <v/>
+      </c>
+      <c r="P6" s="13">
+        <f>Assumptions!P14/365*P4</f>
+        <v/>
+      </c>
+      <c r="Q6" s="13">
+        <f>Assumptions!Q14/365*Q4</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
@@ -14082,6 +16038,18 @@
         <f>Assumptions!N15/365*N5</f>
         <v/>
       </c>
+      <c r="O7" s="13">
+        <f>Assumptions!O15/365*O5</f>
+        <v/>
+      </c>
+      <c r="P7" s="13">
+        <f>Assumptions!P15/365*P5</f>
+        <v/>
+      </c>
+      <c r="Q7" s="13">
+        <f>Assumptions!Q15/365*Q5</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
@@ -14141,6 +16109,18 @@
         <f>Assumptions!N17*N4</f>
         <v/>
       </c>
+      <c r="O8" s="13">
+        <f>Assumptions!O17*O4</f>
+        <v/>
+      </c>
+      <c r="P8" s="13">
+        <f>Assumptions!P17*P4</f>
+        <v/>
+      </c>
+      <c r="Q8" s="13">
+        <f>Assumptions!Q17*Q4</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
@@ -14200,6 +16180,18 @@
         <f>Assumptions!N16/365*N5</f>
         <v/>
       </c>
+      <c r="O9" s="13">
+        <f>Assumptions!O16/365*O5</f>
+        <v/>
+      </c>
+      <c r="P9" s="13">
+        <f>Assumptions!P16/365*P5</f>
+        <v/>
+      </c>
+      <c r="Q9" s="13">
+        <f>Assumptions!Q16/365*Q5</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
@@ -14259,6 +16251,18 @@
         <f>Assumptions!N18*N4</f>
         <v/>
       </c>
+      <c r="O10" s="13">
+        <f>Assumptions!O18*O4</f>
+        <v/>
+      </c>
+      <c r="P10" s="13">
+        <f>Assumptions!P18*P4</f>
+        <v/>
+      </c>
+      <c r="Q10" s="13">
+        <f>Assumptions!Q18*Q4</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -14318,6 +16322,18 @@
         <f>N6+N7+N8-N9-N10</f>
         <v/>
       </c>
+      <c r="O11" s="15">
+        <f>O6+O7+O8-O9-O10</f>
+        <v/>
+      </c>
+      <c r="P11" s="15">
+        <f>P6+P7+P8-P9-P10</f>
+        <v/>
+      </c>
+      <c r="Q11" s="15">
+        <f>Q6+Q7+Q8-Q9-Q10</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
@@ -14373,6 +16389,18 @@
         <f>N11-M11</f>
         <v/>
       </c>
+      <c r="O12" s="13">
+        <f>O11-N11</f>
+        <v/>
+      </c>
+      <c r="P12" s="13">
+        <f>P11-O11</f>
+        <v/>
+      </c>
+      <c r="Q12" s="13">
+        <f>Q11-P11</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -14432,6 +16460,18 @@
         <f>IF(N4=0,"",N6/N4*365)</f>
         <v/>
       </c>
+      <c r="O14" s="32">
+        <f>IF(O4=0,"",O6/O4*365)</f>
+        <v/>
+      </c>
+      <c r="P14" s="32">
+        <f>IF(P4=0,"",P6/P4*365)</f>
+        <v/>
+      </c>
+      <c r="Q14" s="32">
+        <f>IF(Q4=0,"",Q6/Q4*365)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -14491,6 +16531,18 @@
         <f>IF(N5=0,"",N7/N5*365)</f>
         <v/>
       </c>
+      <c r="O15" s="32">
+        <f>IF(O5=0,"",O7/O5*365)</f>
+        <v/>
+      </c>
+      <c r="P15" s="32">
+        <f>IF(P5=0,"",P7/P5*365)</f>
+        <v/>
+      </c>
+      <c r="Q15" s="32">
+        <f>IF(Q5=0,"",Q7/Q5*365)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -14550,6 +16602,18 @@
         <f>IF(N5=0,"",N9/N5*365)</f>
         <v/>
       </c>
+      <c r="O16" s="32">
+        <f>IF(O5=0,"",O9/O5*365)</f>
+        <v/>
+      </c>
+      <c r="P16" s="32">
+        <f>IF(P5=0,"",P9/P5*365)</f>
+        <v/>
+      </c>
+      <c r="Q16" s="32">
+        <f>IF(Q5=0,"",Q9/Q5*365)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="33" t="inlineStr">
@@ -14607,6 +16671,18 @@
       </c>
       <c r="N17" s="34">
         <f>N14+N15-N16</f>
+        <v/>
+      </c>
+      <c r="O17" s="34">
+        <f>O14+O15-O16</f>
+        <v/>
+      </c>
+      <c r="P17" s="34">
+        <f>P14+P15-P16</f>
+        <v/>
+      </c>
+      <c r="Q17" s="34">
+        <f>Q14+Q15-Q16</f>
         <v/>
       </c>
     </row>

</xml_diff>